<commit_message>
Use LBA recruiters[] as "Entreprise cible" proxy for LBB
- jobs[]       → Type "Offre active"     (filtrés par ROME)
- recruiters[] → Type "Entreprise cible" (potentiel embauche tous secteurs)
- "Offre active" prend priorité sur "Entreprise cible" à la dédup
- Sort final pour mettre les "Offre active" en tête avant head(100)
- Result: 17 offres actives + 83 entreprises cibles sur 100 exportées

https://claude.ai/code/session_01XzkQisFxLhzSw3n843fcRb
</commit_message>
<xml_diff>
--- a/entreprises_alternance_paris.xlsx
+++ b/entreprises_alternance_paris.xlsx
@@ -453,12 +453,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="37" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="50" customWidth="1" min="10" max="10"/>
@@ -1092,40 +1092,44 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>85328256400022</t>
+          <t>84311513000018</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>GAVIOTER</t>
+          <t>LES DELICES DE SEVRAN</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>11 boulevard de Sebastopol</t>
+          <t>69 BOULEVARD WESTINGHOUSE</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>75001</t>
+          <t>93270</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr"/>
+          <t>SEVRAN</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>0143516270</t>
+        </is>
+      </c>
       <c r="I13" s="3" t="inlineStr"/>
       <c r="J13" s="3" t="inlineStr"/>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1104</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr"/>
@@ -1143,27 +1147,23 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>82227641600010</t>
+          <t>66202519660347</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>BOULANGERIE BEAUBOURG</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>149 RUE SAINT MARTIN</t>
-        </is>
-      </c>
+          <t>ELIOR RESTAURATION FRANCE</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>92270</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Bois-Colombes</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
@@ -1171,12 +1171,12 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>70.10Z</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1104</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr"/>
@@ -1194,19 +1194,15 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>50843100400037</t>
+          <t>81254993900013</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>DE BELLES MANIERES</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>5 RUE DE TURBIGO</t>
-        </is>
-      </c>
+          <t>SARL LPB</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
           <t>75001</t>
@@ -1214,24 +1210,20 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>0144829271</t>
-        </is>
-      </c>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr"/>
       <c r="J15" s="3" t="inlineStr"/>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1104</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr"/>
@@ -1249,40 +1241,32 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>90428710900014</t>
+          <t>32782338100089</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>ERNEST &amp; VALENTIN RENARD</t>
+          <t>BEAUMARLY</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>5 rue du Renard</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>75004</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>PARIS</t>
-        </is>
-      </c>
+          <t>Paris 75116</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>70.10Z</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1104</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr"/>
@@ -1300,27 +1284,23 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>98136824400019</t>
+          <t>91226424900018</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>BOULANGERIE PATISSERIE PARIS 03</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>34 rue de Montmorency</t>
-        </is>
-      </c>
+          <t>ELIO &amp; FRANCK</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>78100</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Saint-Germain-en-Laye</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr"/>
@@ -1328,12 +1308,12 @@
       <c r="J17" s="3" t="inlineStr"/>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1104</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr"/>
@@ -1351,44 +1331,36 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>55203123900015</t>
+          <t>55204375400019</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>SOCIETE BOULANGERIE SAINT SAUVEUR COLLET</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>100 RUE MONTORGUEIL</t>
-        </is>
-      </c>
+          <t>POTEL ET CHABOT S A</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>75002</t>
+          <t>92310</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>0145080006</t>
-        </is>
-      </c>
+          <t>Sèvres</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>56.21Z</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1104</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr"/>
@@ -1401,27 +1373,27 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>90041114100014</t>
+          <t>85328256400022</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>KAISDIS</t>
+          <t>GAVIOTER</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>42 rue de Turbigo</t>
+          <t>11 boulevard de Sebastopol</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75001</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1452,27 +1424,27 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>80446505200012</t>
+          <t>82227641600010</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>NEW PARK GROUPE</t>
+          <t>BOULANGERIE BEAUBOURG</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>31 rue Dussoubs</t>
+          <t>149 RUE SAINT MARTIN</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>75002</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1485,7 +1457,7 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>4110D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1503,27 +1475,27 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>52288729800019</t>
+          <t>50843100400037</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>MIDORE-REAUMUR</t>
+          <t>DE BELLES MANIERES</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>59 RUE REAUMUR</t>
+          <t>5 RUE DE TURBIGO</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>75002</t>
+          <t>75001</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1531,7 +1503,11 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>0144829271</t>
+        </is>
+      </c>
       <c r="I21" s="3" t="inlineStr"/>
       <c r="J21" s="3" t="inlineStr"/>
       <c r="K21" s="3" t="inlineStr">
@@ -1554,22 +1530,22 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>90507333400013</t>
+          <t>90428710900014</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>LE DIAMANT JAUNE</t>
+          <t>ERNEST &amp; VALENTIN RENARD</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>27 rue des Rosiers</t>
+          <t>5 rue du Renard</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1605,22 +1581,22 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>79768080800012</t>
+          <t>98136824400019</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>SHAYNADIS</t>
+          <t>BOULANGERIE PATISSERIE PARIS 03</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>53 RUE DE TURBIGO</t>
+          <t>34 rue de Montmorency</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1633,16 +1609,12 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>0144788040</t>
-        </is>
-      </c>
+      <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr"/>
       <c r="J23" s="3" t="inlineStr"/>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
@@ -1660,22 +1632,22 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>95365095900018</t>
+          <t>55203123900015</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>ADASHOP</t>
+          <t>SOCIETE BOULANGERIE SAINT SAUVEUR COLLET</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>15 rue de Clery</t>
+          <t>100 RUE MONTORGUEIL</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1688,12 +1660,16 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>0145080006</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -1711,27 +1687,27 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>84304546900015</t>
+          <t>90041114100014</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>LOUIE BOULANGERIE PATISSIERE</t>
+          <t>KAISDIS</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>13 RUE DU PETIT PONT</t>
+          <t>42 rue de Turbigo</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1744,7 +1720,7 @@
       <c r="J25" s="3" t="inlineStr"/>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L25" s="3" t="inlineStr">
@@ -1762,27 +1738,27 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>91162783400011</t>
+          <t>80446505200012</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>LNB PROGRESSION</t>
+          <t>NEW PARK GROUPE</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>5 boulevard Saint Michel</t>
+          <t>31 rue Dussoubs</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75002</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1795,7 +1771,7 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4110D</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -1813,27 +1789,27 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>53524633400051</t>
+          <t>52288729800019</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>OUARIBI DISTRIBUTION</t>
+          <t>MIDORE-REAUMUR</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>18 rue Barbette</t>
+          <t>59 RUE REAUMUR</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75002</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1846,7 +1822,7 @@
       <c r="J27" s="3" t="inlineStr"/>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L27" s="3" t="inlineStr">
@@ -1864,27 +1840,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>95296281900027</t>
+          <t>90507333400013</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>SAINT MARTIN DISTRIBUTION</t>
+          <t>LE DIAMANT JAUNE</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>343 rue Saint Martin</t>
+          <t>27 rue des Rosiers</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75004</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -1897,7 +1873,7 @@
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -1915,27 +1891,27 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>94814278100012</t>
+          <t>79768080800012</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>SYRALIYACOM DISTRIBUTION</t>
+          <t>SHAYNADIS</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>114 boulevard Saint Germain</t>
+          <t>53 RUE DE TURBIGO</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -1943,7 +1919,11 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>0144788040</t>
+        </is>
+      </c>
       <c r="I29" s="3" t="inlineStr"/>
       <c r="J29" s="3" t="inlineStr"/>
       <c r="K29" s="3" t="inlineStr">
@@ -1966,27 +1946,27 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>83218519300014</t>
+          <t>95365095900018</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>ABKH BOULANGERIE</t>
+          <t>ADASHOP</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>351 RUE SAINT MARTIN</t>
+          <t>15 rue de Clery</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75002</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1994,16 +1974,12 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>0656740881</t>
-        </is>
-      </c>
+      <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -2021,27 +1997,27 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>98160217000012</t>
+          <t>84304546900015</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>LE FOURNIL D'AMINE</t>
+          <t>LOUIE BOULANGERIE PATISSIERE</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>351 rue Saint Martin</t>
+          <t>13 RUE DU PETIT PONT</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -2072,27 +2048,27 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>88378730100018</t>
+          <t>91162783400011</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>AUX DESIRS DE MANON</t>
+          <t>LNB PROGRESSION</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>129 rue Saint Antoine</t>
+          <t>5 boulevard Saint Michel</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>75004</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2123,27 +2099,27 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>44028375208195</t>
+          <t>53524633400051</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>CSF</t>
+          <t>OUARIBI DISTRIBUTION</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>79 RUE DE SEINE</t>
+          <t>18 rue Barbette</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -2174,22 +2150,22 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>91514335800017</t>
+          <t>95296281900027</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>LT2G</t>
+          <t>SAINT MARTIN DISTRIBUTION</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>183 RUE DU TEMPLE</t>
+          <t>343 rue Saint Martin</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -2202,16 +2178,12 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>0134697793</t>
-        </is>
-      </c>
+      <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -2229,27 +2201,27 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>84396530200014</t>
+          <t>94814278100012</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>LNB DEVELOPPEMENT</t>
+          <t>SYRALIYACOM DISTRIBUTION</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>359 RUE SAINT MARTIN</t>
+          <t>114 boulevard Saint Germain</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -2262,7 +2234,7 @@
       <c r="J35" s="3" t="inlineStr"/>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
@@ -2280,27 +2252,27 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>89288269700014</t>
+          <t>83218519300014</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>ATELIER BABKA ZANA</t>
+          <t>ABKH BOULANGERIE</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>5 rue des Colonnes</t>
+          <t>351 RUE SAINT MARTIN</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>75002</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -2308,7 +2280,11 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>0656740881</t>
+        </is>
+      </c>
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr">
@@ -2331,27 +2307,27 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>48402650500038</t>
+          <t>98160217000012</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>la pelle a bois</t>
+          <t>LE FOURNIL D'AMINE</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>149 RUE MONTMARTRE</t>
+          <t>351 rue Saint Martin</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>75002</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -2382,27 +2358,27 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>98105235000015</t>
+          <t>88378730100018</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>LUMDYS</t>
+          <t>AUX DESIRS DE MANON</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>8 rue du faubourg Saint Martin</t>
+          <t>129 rue Saint Antoine</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75004</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2415,7 +2391,7 @@
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -2433,27 +2409,27 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>89490730200018</t>
+          <t>44028375208195</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>PETIT FOURNIL</t>
+          <t>CSF</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>6 rue Rameau</t>
+          <t>79 RUE DE SEINE</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>75002</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -2466,7 +2442,7 @@
       <c r="J39" s="3" t="inlineStr"/>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L39" s="3" t="inlineStr">
@@ -2484,27 +2460,27 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>79514622400055</t>
+          <t>91514335800017</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>ILANDAN</t>
+          <t>LT2G</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>43 boulevard Saint Germain</t>
+          <t>183 RUE DU TEMPLE</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2512,12 +2488,16 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>0134697793</t>
+        </is>
+      </c>
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -2535,27 +2515,27 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>34326262213928</t>
+          <t>84396530200014</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>LIDL</t>
+          <t>LNB DEVELOPPEMENT</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>8 boulevard de Strasbourg</t>
+          <t>359 RUE SAINT MARTIN</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -2568,7 +2548,7 @@
       <c r="J41" s="3" t="inlineStr"/>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr">
@@ -2586,27 +2566,27 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>32930252500020</t>
+          <t>89288269700014</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>MAISON MULOT SAS</t>
+          <t>ATELIER BABKA ZANA</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>76 RUE DE SEINE</t>
+          <t>5 rue des Colonnes</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>75002</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2614,11 +2594,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>0143268577</t>
-        </is>
-      </c>
+      <c r="H42" s="2" t="inlineStr"/>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr">
@@ -2641,27 +2617,27 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>84166072300013</t>
+          <t>48402650500038</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>LP PROD</t>
+          <t>la pelle a bois</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>12 rue du faubourg Poissonniere</t>
+          <t>149 RUE MONTMARTRE</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75002</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -2669,11 +2645,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>0142385509</t>
-        </is>
-      </c>
+      <c r="H43" s="3" t="inlineStr"/>
       <c r="I43" s="3" t="inlineStr"/>
       <c r="J43" s="3" t="inlineStr"/>
       <c r="K43" s="3" t="inlineStr">
@@ -2696,27 +2668,27 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>81187718200022</t>
+          <t>98105235000015</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>SODIGERMAIN</t>
+          <t>LUMDYS</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>14 rue Lobineau</t>
+          <t>8 rue du faubourg Saint Martin</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2747,27 +2719,27 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>90162631700019</t>
+          <t>89490730200018</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>MAISON ISLAND</t>
+          <t>PETIT FOURNIL</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>8 rue des Filles du Calvaire</t>
+          <t>6 rue Rameau</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75002</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -2775,11 +2747,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>0647915566</t>
-        </is>
-      </c>
+      <c r="H45" s="3" t="inlineStr"/>
       <c r="I45" s="3" t="inlineStr"/>
       <c r="J45" s="3" t="inlineStr"/>
       <c r="K45" s="3" t="inlineStr">
@@ -2802,27 +2770,27 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>45045418600013</t>
+          <t>79514622400055</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>COFIGILLES</t>
+          <t>ILANDAN</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>24 RUE SAINT GILLES</t>
+          <t>43 boulevard Saint Germain</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -2830,11 +2798,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>0967452096</t>
-        </is>
-      </c>
+      <c r="H46" s="2" t="inlineStr"/>
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr">
@@ -2857,27 +2821,27 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>94940810800015</t>
+          <t>34326262213928</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>MELDES</t>
+          <t>LIDL</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>9 rue du faubourg Montmartre</t>
+          <t>8 boulevard de Strasbourg</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -2908,22 +2872,22 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>55208329701430</t>
+          <t>32930252500020</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
+          <t>MAISON MULOT SAS</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>7 RUE DU DRAGON</t>
+          <t>76 RUE DE SEINE</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -2938,14 +2902,14 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>0145481808</t>
+          <t>0143268577</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
@@ -2963,27 +2927,27 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>88860572200014</t>
+          <t>84166072300013</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>DISTRIMICHEL</t>
+          <t>LP PROD</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>55 boulevard Saint Michel</t>
+          <t>12 rue du faubourg Poissonniere</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -2991,12 +2955,16 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H49" s="3" t="inlineStr"/>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>0142385509</t>
+        </is>
+      </c>
       <c r="I49" s="3" t="inlineStr"/>
       <c r="J49" s="3" t="inlineStr"/>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr">
@@ -3014,27 +2982,27 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>88536923100034</t>
+          <t>81187718200022</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>ROULES BOULES</t>
+          <t>SODIGERMAIN</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>1B rue Saint Gilles</t>
+          <t>14 rue Lobineau</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -3047,7 +3015,7 @@
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
@@ -3065,27 +3033,27 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>75198013700028</t>
+          <t>90162631700019</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>TAL</t>
+          <t>MAISON ISLAND</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>29 RUE SAINT ANTOINE</t>
+          <t>8 rue des Filles du Calvaire</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>75004</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -3095,7 +3063,7 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>0235489596</t>
+          <t>0647915566</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr"/>
@@ -3120,22 +3088,22 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>89288269700022</t>
+          <t>45045418600013</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>ATELIER BABKA ZANA</t>
+          <t>COFIGILLES</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>8 RUE DU PAS DE LA MULE</t>
+          <t>24 RUE SAINT GILLES</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -3148,12 +3116,16 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>0967452096</t>
+        </is>
+      </c>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
@@ -3171,22 +3143,22 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>33496216400011</t>
+          <t>94940810800015</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>SOGIBERGERE</t>
+          <t>MELDES</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>5 RUE GEOFFROY MARIE</t>
+          <t>9 rue du faubourg Montmartre</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
@@ -3199,11 +3171,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H53" s="3" t="inlineStr">
-        <is>
-          <t>0142463633</t>
-        </is>
-      </c>
+      <c r="H53" s="3" t="inlineStr"/>
       <c r="I53" s="3" t="inlineStr"/>
       <c r="J53" s="3" t="inlineStr"/>
       <c r="K53" s="3" t="inlineStr">
@@ -3226,27 +3194,27 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>50449677900043</t>
+          <t>55208329701430</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>VAUGIDARD DISTRIBUTION</t>
+          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>18 rue SOUFFLOT</t>
+          <t>7 RUE DU DRAGON</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -3254,7 +3222,11 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>0145481808</t>
+        </is>
+      </c>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr">
@@ -3277,27 +3249,27 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>38765154000024</t>
+          <t>88860572200014</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>SOGIQUATRE</t>
+          <t>DISTRIMICHEL</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>17 boulevard Henri IV</t>
+          <t>55 boulevard Saint Michel</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>75004</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -3328,27 +3300,27 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>52022307400037</t>
+          <t>88536923100034</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>LE PETIT MITRON</t>
+          <t>ROULES BOULES</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>8 rue Oberkampf</t>
+          <t>1B rue Saint Gilles</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -3356,11 +3328,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>0145411655</t>
-        </is>
-      </c>
+      <c r="H56" s="2" t="inlineStr"/>
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="2" t="inlineStr">
@@ -3383,27 +3351,27 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>90947551900015</t>
+          <t>75198013700028</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>SP MARSEILLE</t>
+          <t>TAL</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>14 RUE RICHER</t>
+          <t>29 RUE SAINT ANTOINE</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75004</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -3411,7 +3379,11 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H57" s="3" t="inlineStr"/>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>0235489596</t>
+        </is>
+      </c>
       <c r="I57" s="3" t="inlineStr"/>
       <c r="J57" s="3" t="inlineStr"/>
       <c r="K57" s="3" t="inlineStr">
@@ -3434,27 +3406,27 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>44380979300021</t>
+          <t>89288269700022</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>AU BLE D'OR</t>
+          <t>ATELIER BABKA ZANA</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>23 BOULEVARD VOLTAIRE</t>
+          <t>8 RUE DU PAS DE LA MULE</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -3485,22 +3457,22 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>80403394200017</t>
+          <t>33496216400011</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>LES DELICES DE LAFAYETTE</t>
+          <t>SOGIBERGERE</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>1 rue de Provence</t>
+          <t>5 RUE GEOFFROY MARIE</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
@@ -3515,14 +3487,14 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>0153340875</t>
+          <t>0142463633</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr"/>
       <c r="J59" s="3" t="inlineStr"/>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
@@ -3540,27 +3512,27 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>82315851400021</t>
+          <t>50449677900043</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>CITY RENNES</t>
+          <t>VAUGIDARD DISTRIBUTION</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>71 RUE DE RENNES</t>
+          <t>18 rue SOUFFLOT</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -3591,27 +3563,27 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>83464080700014</t>
+          <t>38765154000024</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>LES FOURNILS DE GAIA</t>
+          <t>SOGIQUATRE</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>28 BOULEVARD VOLTAIRE</t>
+          <t>17 boulevard Henri IV</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75004</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -3624,7 +3596,7 @@
       <c r="J61" s="3" t="inlineStr"/>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L61" s="3" t="inlineStr">
@@ -3642,27 +3614,27 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>88406515200016</t>
+          <t>52022307400037</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>VDB</t>
+          <t>LE PETIT MITRON</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>12 rue Cadet</t>
+          <t>8 rue Oberkampf</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -3670,7 +3642,11 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>0145411655</t>
+        </is>
+      </c>
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="2" t="inlineStr">
@@ -3693,27 +3669,27 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>80302565900019</t>
+          <t>90947551900015</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>LE TEMPS DU REVE</t>
+          <t>SP MARSEILLE</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>20 RUE JEAN PIERRE TIMBAUD</t>
+          <t>14 RUE RICHER</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -3721,11 +3697,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H63" s="3" t="inlineStr">
-        <is>
-          <t>0982507448</t>
-        </is>
-      </c>
+      <c r="H63" s="3" t="inlineStr"/>
       <c r="I63" s="3" t="inlineStr"/>
       <c r="J63" s="3" t="inlineStr"/>
       <c r="K63" s="3" t="inlineStr">
@@ -3748,27 +3720,27 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>49862034300034</t>
+          <t>44380979300021</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>DISTRIBLANCHE</t>
+          <t>AU BLE D'OR</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>9 RUE LE GOFF</t>
+          <t>23 BOULEVARD VOLTAIRE</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -3781,7 +3753,7 @@
       <c r="J64" s="2" t="inlineStr"/>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
@@ -3799,27 +3771,27 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>88922904300019</t>
+          <t>80403394200017</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>DISTRI-BASTILLE</t>
+          <t>LES DELICES DE LAFAYETTE</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>5 boulevard Beaumarchais</t>
+          <t>1 rue de Provence</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>75004</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
@@ -3827,12 +3799,16 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H65" s="3" t="inlineStr"/>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>0153340875</t>
+        </is>
+      </c>
       <c r="I65" s="3" t="inlineStr"/>
       <c r="J65" s="3" t="inlineStr"/>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L65" s="3" t="inlineStr">
@@ -3850,27 +3826,27 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>92239334300012</t>
+          <t>82315851400021</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>PARIS AGRO DISTRIB</t>
+          <t>CITY RENNES</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>63 rue d Hauteville</t>
+          <t>71 RUE DE RENNES</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -3901,27 +3877,27 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>79124664800012</t>
+          <t>83464080700014</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>SARL RENNES 81</t>
+          <t>LES FOURNILS DE GAIA</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>81 RUE DE RENNES</t>
+          <t>28 BOULEVARD VOLTAIRE</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G67" s="3" t="inlineStr">
@@ -3929,11 +3905,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H67" s="3" t="inlineStr">
-        <is>
-          <t>0620474041</t>
-        </is>
-      </c>
+      <c r="H67" s="3" t="inlineStr"/>
       <c r="I67" s="3" t="inlineStr"/>
       <c r="J67" s="3" t="inlineStr"/>
       <c r="K67" s="3" t="inlineStr">
@@ -3956,27 +3928,27 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>83387850700031</t>
+          <t>88406515200016</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>ALVIDIS</t>
+          <t>VDB</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>20 RUE DU CHEMIN VERT</t>
+          <t>12 rue Cadet</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -3989,7 +3961,7 @@
       <c r="J68" s="2" t="inlineStr"/>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
@@ -4007,27 +3979,27 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>42178748200023</t>
+          <t>80302565900019</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>SNC LILLE BELLECHASSE</t>
+          <t>LE TEMPS DU REVE</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>97 rue de Lille</t>
+          <t>20 RUE JEAN PIERRE TIMBAUD</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>75007</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -4035,12 +4007,16 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H69" s="3" t="inlineStr"/>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>0982507448</t>
+        </is>
+      </c>
       <c r="I69" s="3" t="inlineStr"/>
       <c r="J69" s="3" t="inlineStr"/>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>4110D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L69" s="3" t="inlineStr">
@@ -4058,27 +4034,27 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>88232661400022</t>
+          <t>49862034300034</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>SLBC</t>
+          <t>DISTRIBLANCHE</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>92 boulevard Richard Lenoir</t>
+          <t>9 RUE LE GOFF</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -4109,27 +4085,27 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>81355955600028</t>
+          <t>88922904300019</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>LACETOP</t>
+          <t>DISTRI-BASTILLE</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>37 RUE LACEPEDE</t>
+          <t>5 boulevard Beaumarchais</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75004</t>
         </is>
       </c>
       <c r="G71" s="3" t="inlineStr">
@@ -4160,27 +4136,27 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>52755379600014</t>
+          <t>92239334300012</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>MONTHOLON DIS</t>
+          <t>PARIS AGRO DISTRIB</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>88 RUE LA FAYETTE</t>
+          <t>63 rue d Hauteville</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -4211,22 +4187,22 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>75237791100017</t>
+          <t>79124664800012</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>REINE</t>
+          <t>SARL RENNES 81</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>101 RUE DE RENNES</t>
+          <t>81 RUE DE RENNES</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
@@ -4239,7 +4215,11 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H73" s="3" t="inlineStr"/>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>0620474041</t>
+        </is>
+      </c>
       <c r="I73" s="3" t="inlineStr"/>
       <c r="J73" s="3" t="inlineStr"/>
       <c r="K73" s="3" t="inlineStr">
@@ -4262,27 +4242,27 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>90236206000011</t>
+          <t>83387850700031</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>ATELIER LINNE</t>
+          <t>ALVIDIS</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>6 rue Linne</t>
+          <t>20 RUE DU CHEMIN VERT</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -4295,7 +4275,7 @@
       <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr">
@@ -4313,27 +4293,27 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>82933786400021</t>
+          <t>42178748200023</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>LPJ 12</t>
+          <t>SNC LILLE BELLECHASSE</t>
         </is>
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>248 RUE SAINT JACQUES</t>
+          <t>97 rue de Lille</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75007</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -4346,7 +4326,7 @@
       <c r="J75" s="3" t="inlineStr"/>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4110D</t>
         </is>
       </c>
       <c r="L75" s="3" t="inlineStr">
@@ -4364,27 +4344,27 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>79275981300019</t>
+          <t>88232661400022</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>BOULANGERIE DE VARENNE</t>
+          <t>SLBC</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>31 RUE DE VARENNE</t>
+          <t>92 boulevard Richard Lenoir</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>75007</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -4397,7 +4377,7 @@
       <c r="J76" s="2" t="inlineStr"/>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L76" s="2" t="inlineStr">
@@ -4415,27 +4395,27 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>89829090300019</t>
+          <t>81355955600028</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>LIBERTE MAUBEUGE</t>
+          <t>LACETOP</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>1 rue Hippolyte Lebas</t>
+          <t>37 RUE LACEPEDE</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
@@ -4448,7 +4428,7 @@
       <c r="J77" s="3" t="inlineStr"/>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L77" s="3" t="inlineStr">
@@ -4466,27 +4446,27 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>91004295100020</t>
+          <t>52755379600014</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>MIE MIE</t>
+          <t>MONTHOLON DIS</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>25 rue Sedaine</t>
+          <t>88 RUE LA FAYETTE</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4499,7 +4479,7 @@
       <c r="J78" s="2" t="inlineStr"/>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
@@ -4517,27 +4497,27 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>90469185400023</t>
+          <t>75237791100017</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>LA COURONNEE</t>
+          <t>REINE</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>4 place Franz Liszt</t>
+          <t>101 RUE DE RENNES</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -4568,22 +4548,22 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>82200690400012</t>
+          <t>90236206000011</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>L'ATELIER DE MONGE</t>
+          <t>ATELIER LINNE</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>48 RUE DE LA CLEF</t>
+          <t>6 rue Linne</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -4619,27 +4599,27 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>81012935300035</t>
+          <t>82933786400021</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>LE PAIN RETROUVE</t>
+          <t>LPJ 12</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>18 RUE DES MARTYRS</t>
+          <t>248 RUE SAINT JACQUES</t>
         </is>
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -4647,11 +4627,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H81" s="3" t="inlineStr">
-        <is>
-          <t>0753210804</t>
-        </is>
-      </c>
+      <c r="H81" s="3" t="inlineStr"/>
       <c r="I81" s="3" t="inlineStr"/>
       <c r="J81" s="3" t="inlineStr"/>
       <c r="K81" s="3" t="inlineStr">
@@ -4674,27 +4650,27 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>53159116200015</t>
+          <t>79275981300019</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>LES DELICES DES FAUBOURGS</t>
+          <t>BOULANGERIE DE VARENNE</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>156 DU FAUBOURG SAINT MARTIN</t>
+          <t>31 RUE DE VARENNE</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75007</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -4702,11 +4678,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>0698011212</t>
-        </is>
-      </c>
+      <c r="H82" s="2" t="inlineStr"/>
       <c r="I82" s="2" t="inlineStr"/>
       <c r="J82" s="2" t="inlineStr"/>
       <c r="K82" s="2" t="inlineStr">
@@ -4729,27 +4701,27 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>79207221700013</t>
+          <t>89829090300019</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>MAISON COUPINOT</t>
+          <t>LIBERTE MAUBEUGE</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>88T AVENUE PARMENTIER</t>
+          <t>1 rue Hippolyte Lebas</t>
         </is>
       </c>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G83" s="3" t="inlineStr">
@@ -4780,22 +4752,22 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>91904841300018</t>
+          <t>91004295100020</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>LE FOURNIL DE LA ROQUETTE</t>
+          <t>MIE MIE</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>53 rue de la Roquette</t>
+          <t>25 rue Sedaine</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -4831,27 +4803,27 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>49323098100042</t>
+          <t>90469185400023</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>MAISON SEO</t>
+          <t>LA COURONNEE</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>32 RUE SAINT PLACIDE</t>
+          <t>4 place Franz Liszt</t>
         </is>
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -4882,27 +4854,27 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>55208329701588</t>
+          <t>82200690400012</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
+          <t>L'ATELIER DE MONGE</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>52 RUE DE CAUMARTIN</t>
+          <t>48 RUE DE LA CLEF</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -4910,16 +4882,12 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H86" s="2" t="inlineStr">
-        <is>
-          <t>0144537979</t>
-        </is>
-      </c>
+      <c r="H86" s="2" t="inlineStr"/>
       <c r="I86" s="2" t="inlineStr"/>
       <c r="J86" s="2" t="inlineStr"/>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L86" s="2" t="inlineStr">
@@ -4937,22 +4905,22 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>44356204600047</t>
+          <t>81012935300035</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>LES GOURMANDISES DE SAINT LAZARE</t>
+          <t>LE PAIN RETROUVE</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>71 RUE SAINT LAZARE</t>
+          <t>18 RUE DES MARTYRS</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
@@ -4965,7 +4933,11 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H87" s="3" t="inlineStr"/>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>0753210804</t>
+        </is>
+      </c>
       <c r="I87" s="3" t="inlineStr"/>
       <c r="J87" s="3" t="inlineStr"/>
       <c r="K87" s="3" t="inlineStr">
@@ -4988,27 +4960,27 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>98137478800017</t>
+          <t>53159116200015</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>BAKERY 8</t>
+          <t>LES DELICES DES FAUBOURGS</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>8 rue de Charonne</t>
+          <t>156 DU FAUBOURG SAINT MARTIN</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -5016,7 +4988,11 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>0698011212</t>
+        </is>
+      </c>
       <c r="I88" s="2" t="inlineStr"/>
       <c r="J88" s="2" t="inlineStr"/>
       <c r="K88" s="2" t="inlineStr">
@@ -5039,27 +5015,27 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>88035775100010</t>
+          <t>79207221700013</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>BOULANGERIE HADDAG</t>
+          <t>MAISON COUPINOT</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>21 rue Condorcet</t>
+          <t>88T AVENUE PARMENTIER</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
@@ -5090,27 +5066,27 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>91515182300019</t>
+          <t>91904841300018</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>AUX 9 BLES D'OR</t>
+          <t>LE FOURNIL DE LA ROQUETTE</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>21 RUE CONDORCET</t>
+          <t>53 rue de la Roquette</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -5141,27 +5117,27 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>52750734700021</t>
+          <t>49323098100042</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>SAINT LAZARE DISTRIBUTION</t>
+          <t>MAISON SEO</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>81 rue Saint Lazare</t>
+          <t>32 RUE SAINT PLACIDE</t>
         </is>
       </c>
       <c r="F91" s="3" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G91" s="3" t="inlineStr">
@@ -5174,7 +5150,7 @@
       <c r="J91" s="3" t="inlineStr"/>
       <c r="K91" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L91" s="3" t="inlineStr">
@@ -5192,27 +5168,27 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>80090315500011</t>
+          <t>55208329701588</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>SANG L.L</t>
+          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>235 RUE DE BERCY</t>
+          <t>52 RUE DE CAUMARTIN</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>75012</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -5220,12 +5196,16 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H92" s="2" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>0144537979</t>
+        </is>
+      </c>
       <c r="I92" s="2" t="inlineStr"/>
       <c r="J92" s="2" t="inlineStr"/>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L92" s="2" t="inlineStr">
@@ -5243,27 +5223,27 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>84186128900012</t>
+          <t>44356204600047</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>ATELIER GUINOT BAKER</t>
+          <t>LES GOURMANDISES DE SAINT LAZARE</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>6 RUE SAINT AMBROISE</t>
+          <t>71 RUE SAINT LAZARE</t>
         </is>
       </c>
       <c r="F93" s="3" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G93" s="3" t="inlineStr">
@@ -5271,11 +5251,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H93" s="3" t="inlineStr">
-        <is>
-          <t>0662415274</t>
-        </is>
-      </c>
+      <c r="H93" s="3" t="inlineStr"/>
       <c r="I93" s="3" t="inlineStr"/>
       <c r="J93" s="3" t="inlineStr"/>
       <c r="K93" s="3" t="inlineStr">
@@ -5298,27 +5274,27 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>53881702400010</t>
+          <t>98137478800017</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>HOUIRES TAHAR</t>
+          <t>BAKERY 8</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>215 RUE SAINT MAUR</t>
+          <t>8 rue de Charonne</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -5326,11 +5302,7 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H94" s="2" t="inlineStr">
-        <is>
-          <t>0607463025</t>
-        </is>
-      </c>
+      <c r="H94" s="2" t="inlineStr"/>
       <c r="I94" s="2" t="inlineStr"/>
       <c r="J94" s="2" t="inlineStr"/>
       <c r="K94" s="2" t="inlineStr">
@@ -5353,32 +5325,32 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>92225689600015</t>
+          <t>88035775100010</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>PAIN DU FAUBOURG</t>
+          <t>BOULANGERIE HADDAG</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>97 Rue du Faubourg du Temple</t>
+          <t>21 rue Condorcet</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr"/>
@@ -5404,27 +5376,27 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>92044574900012</t>
+          <t>91515182300019</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>LIBERTE MOUFFETARD</t>
+          <t>AUX 9 BLES D'OR</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>119 rue Mouffetard</t>
+          <t>21 RUE CONDORCET</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -5455,22 +5427,22 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>88519655000028</t>
+          <t>52750734700021</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>TURGODIS</t>
+          <t>SAINT LAZARE DISTRIBUTION</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>61 rue Marguerite de Rochechouart</t>
+          <t>81 rue Saint Lazare</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
@@ -5506,27 +5478,27 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>72205443400013</t>
+          <t>80090315500011</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>A LA BONNE SOURCE</t>
+          <t>SANG L.L</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>122 RUE MOUFFETARD</t>
+          <t>235 RUE DE BERCY</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75012</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -5534,16 +5506,12 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H98" s="2" t="inlineStr">
-        <is>
-          <t>0143312963</t>
-        </is>
-      </c>
+      <c r="H98" s="2" t="inlineStr"/>
       <c r="I98" s="2" t="inlineStr"/>
       <c r="J98" s="2" t="inlineStr"/>
       <c r="K98" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L98" s="2" t="inlineStr">
@@ -5561,22 +5529,22 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>85327274800015</t>
+          <t>84186128900012</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>SASU BLE &amp; MIEL</t>
+          <t>ATELIER GUINOT BAKER</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>81 RUE DE LA ROQUETTE</t>
+          <t>6 RUE SAINT AMBROISE</t>
         </is>
       </c>
       <c r="F99" s="3" t="inlineStr">
@@ -5589,7 +5557,11 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H99" s="3" t="inlineStr"/>
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>0662415274</t>
+        </is>
+      </c>
       <c r="I99" s="3" t="inlineStr"/>
       <c r="J99" s="3" t="inlineStr"/>
       <c r="K99" s="3" t="inlineStr">
@@ -5612,27 +5584,27 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>82261320400012</t>
+          <t>53881702400010</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>AUX DELICES DE GARE DE LYON</t>
+          <t>HOUIRES TAHAR</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>23 rue DE LYON</t>
+          <t>215 RUE SAINT MAUR</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>75012</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -5640,7 +5612,11 @@
           <t>PARIS</t>
         </is>
       </c>
-      <c r="H100" s="2" t="inlineStr"/>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>0607463025</t>
+        </is>
+      </c>
       <c r="I100" s="2" t="inlineStr"/>
       <c r="J100" s="2" t="inlineStr"/>
       <c r="K100" s="2" t="inlineStr">
@@ -5663,22 +5639,22 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Offre active</t>
+          <t>Entreprise cible</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>83254766500014</t>
+          <t>92225689600015</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>SARL BRUMANO</t>
+          <t>PAIN DU FAUBOURG</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>83 RUE DE MAUBEUGE</t>
+          <t>97 Rue du Faubourg du Temple</t>
         </is>
       </c>
       <c r="F101" s="3" t="inlineStr">
@@ -5688,14 +5664,10 @@
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
-        </is>
-      </c>
-      <c r="H101" s="3" t="inlineStr">
-        <is>
-          <t>0630321473</t>
-        </is>
-      </c>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="H101" s="3" t="inlineStr"/>
       <c r="I101" s="3" t="inlineStr"/>
       <c r="J101" s="3" t="inlineStr"/>
       <c r="K101" s="3" t="inlineStr">
@@ -5758,7 +5730,7 @@
         </is>
       </c>
       <c r="B107" s="4" t="n">
-        <v>100</v>
+        <v>17</v>
       </c>
     </row>
     <row r="108">
@@ -5768,7 +5740,7 @@
         </is>
       </c>
       <c r="B108" s="4" t="n">
-        <v>0</v>
+        <v>83</v>
       </c>
     </row>
     <row r="109">
@@ -5778,7 +5750,7 @@
         </is>
       </c>
       <c r="B109" s="4" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Export 150 LBA contacts to Excel
Increase MAX_TOTAL from 100 to 150.
Result: 17 offres actives + 133 entreprises cibles (215 uniques disponibles).

https://claude.ai/code/session_01XzkQisFxLhzSw3n843fcRb
</commit_message>
<xml_diff>
--- a/entreprises_alternance_paris.xlsx
+++ b/entreprises_alternance_paris.xlsx
@@ -449,14 +449,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M109"/>
+  <dimension ref="A1:M159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="25" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
@@ -5682,75 +5682,2665 @@
       </c>
       <c r="M101" s="3" t="inlineStr"/>
     </row>
-    <row r="102"/>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>92044574900012</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>LIBERTE MOUFFETARD</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>119 rue Mouffetard</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>75005</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr"/>
+      <c r="I102" s="2" t="inlineStr"/>
+      <c r="J102" s="2" t="inlineStr"/>
+      <c r="K102" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M102" s="2" t="inlineStr"/>
+    </row>
     <row r="103">
-      <c r="A103" s="4" t="inlineStr">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>88519655000028</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>TURGODIS</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>61 rue Marguerite de Rochechouart</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="G103" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H103" s="3" t="inlineStr"/>
+      <c r="I103" s="3" t="inlineStr"/>
+      <c r="J103" s="3" t="inlineStr"/>
+      <c r="K103" s="3" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L103" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M103" s="3" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>72205443400013</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>A LA BONNE SOURCE</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>122 RUE MOUFFETARD</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>75005</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>0143312963</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr"/>
+      <c r="J104" s="2" t="inlineStr"/>
+      <c r="K104" s="2" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>85327274800015</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>SASU BLE &amp; MIEL</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>81 RUE DE LA ROQUETTE</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="G105" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H105" s="3" t="inlineStr"/>
+      <c r="I105" s="3" t="inlineStr"/>
+      <c r="J105" s="3" t="inlineStr"/>
+      <c r="K105" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L105" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M105" s="3" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>82261320400012</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>AUX DELICES DE GARE DE LYON</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>23 rue DE LYON</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>75012</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr"/>
+      <c r="I106" s="2" t="inlineStr"/>
+      <c r="J106" s="2" t="inlineStr"/>
+      <c r="K106" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M106" s="2" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>83254766500014</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>SARL BRUMANO</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>83 RUE DE MAUBEUGE</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>75010</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H107" s="3" t="inlineStr">
+        <is>
+          <t>0630321473</t>
+        </is>
+      </c>
+      <c r="I107" s="3" t="inlineStr"/>
+      <c r="J107" s="3" t="inlineStr"/>
+      <c r="K107" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L107" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M107" s="3" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>92009368900015</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>LMRV</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>37 rue Claude Bernard</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>75005</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr"/>
+      <c r="I108" s="2" t="inlineStr"/>
+      <c r="J108" s="2" t="inlineStr"/>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>52397305500016</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>LA BOULANGERIE DE JEANNE</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>109 AVENUE LEDRU ROLLIN</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H109" s="3" t="inlineStr"/>
+      <c r="I109" s="3" t="inlineStr"/>
+      <c r="J109" s="3" t="inlineStr"/>
+      <c r="K109" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L109" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M109" s="3" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>83518647900019</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>MAISON AURELIE RIBAY</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>36B RUE DE DUNKERQUE</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>75010</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr"/>
+      <c r="I110" s="2" t="inlineStr"/>
+      <c r="J110" s="2" t="inlineStr"/>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>95396171100017</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>LE FOURNIL DE DANY ET LEO</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>12 avenue Parmentier</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H111" s="3" t="inlineStr"/>
+      <c r="I111" s="3" t="inlineStr"/>
+      <c r="J111" s="3" t="inlineStr"/>
+      <c r="K111" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L111" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M111" s="3" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>80430576100012</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>DAR SALEM</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>11 RUE DE SAMBRE ET MEUSE</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>75010</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr"/>
+      <c r="I112" s="2" t="inlineStr"/>
+      <c r="J112" s="2" t="inlineStr"/>
+      <c r="K112" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L112" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M112" s="2" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>92161760100015</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>LE FOURNIL DU 5EME</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>22 boulevard de l Hopital</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>75005</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr"/>
+      <c r="I113" s="3" t="inlineStr"/>
+      <c r="J113" s="3" t="inlineStr"/>
+      <c r="K113" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L113" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M113" s="3" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>90448541400018</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>LEONIE SACRE COEUR</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>15 avenue Trudaine</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr"/>
+      <c r="I114" s="2" t="inlineStr"/>
+      <c r="J114" s="2" t="inlineStr"/>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M114" s="2" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>81000098400031</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>NADIMAR DISTRIBUTION</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>24 RUE DE LA GRANGE AUX BELLES</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>75010</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H115" s="3" t="inlineStr"/>
+      <c r="I115" s="3" t="inlineStr"/>
+      <c r="J115" s="3" t="inlineStr"/>
+      <c r="K115" s="3" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L115" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M115" s="3" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>89751484000015</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>BASCIU &amp; BELANGE</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>151B boulevard du Montparnasse</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>75006</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr"/>
+      <c r="I116" s="2" t="inlineStr"/>
+      <c r="J116" s="2" t="inlineStr"/>
+      <c r="K116" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M116" s="2" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr">
+        <is>
+          <t>88285102500016</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>LE TEMPS D'UNE GOURMANDISE</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>94 boulevard de Port Royal</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>75005</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="inlineStr"/>
+      <c r="I117" s="3" t="inlineStr"/>
+      <c r="J117" s="3" t="inlineStr"/>
+      <c r="K117" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L117" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M117" s="3" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>40174230900024</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>BOULANGERIE DE SEVRES</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>54 RUE DE SEVRES</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>75007</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>0147833040</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr"/>
+      <c r="J118" s="2" t="inlineStr"/>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M118" s="2" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>50234606700015</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>sarl p s v a</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>1 RUE MICHEL CHASLES</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>75012</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H119" s="3" t="inlineStr"/>
+      <c r="I119" s="3" t="inlineStr"/>
+      <c r="J119" s="3" t="inlineStr"/>
+      <c r="K119" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L119" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M119" s="3" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>82754610200027</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>S.A.P.P SOCIETE ARTISANS PATISSIERS PA</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>5 RUE DELAMBRE 5 7</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>75014</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr"/>
+      <c r="I120" s="2" t="inlineStr"/>
+      <c r="J120" s="2" t="inlineStr"/>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M120" s="2" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>49833396200039</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>MIDORE BONAPARTE</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>40 rue de Londres</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H121" s="3" t="inlineStr"/>
+      <c r="I121" s="3" t="inlineStr"/>
+      <c r="J121" s="3" t="inlineStr"/>
+      <c r="K121" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L121" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M121" s="3" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>80348700800028</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>SARLU AUX DELICES DE LOLO</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>92 avenue de la Republique</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>0148057385</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr"/>
+      <c r="J122" s="2" t="inlineStr"/>
+      <c r="K122" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L122" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M122" s="2" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>35088924200011</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>SUPER DELAMBRE</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>11 rue Delambre</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>75014</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>0142790787</t>
+        </is>
+      </c>
+      <c r="I123" s="3" t="inlineStr"/>
+      <c r="J123" s="3" t="inlineStr"/>
+      <c r="K123" s="3" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L123" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M123" s="3" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>90400197100020</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>WYNWOOD BAKERY</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>207 rue du faubourg Saint Martin</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>75010</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr"/>
+      <c r="I124" s="2" t="inlineStr"/>
+      <c r="J124" s="2" t="inlineStr"/>
+      <c r="K124" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L124" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M124" s="2" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>82234103800013</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>BOULANGERIE SAINT ANTOINE</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>153 Rue du Faubourg Saint-Antoine</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="H125" s="3" t="inlineStr">
+        <is>
+          <t>0143077758</t>
+        </is>
+      </c>
+      <c r="I125" s="3" t="inlineStr"/>
+      <c r="J125" s="3" t="inlineStr"/>
+      <c r="K125" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L125" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M125" s="3" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>88071932300029</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>LAUREDIS</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>16B rue Pierre Fontaine</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>0611324848</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr"/>
+      <c r="J126" s="2" t="inlineStr"/>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L126" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M126" s="2" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>82831040900028</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>BV DIS</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>114 BOULEVARD DE BELLEVILLE</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>75020</t>
+        </is>
+      </c>
+      <c r="G127" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H127" s="3" t="inlineStr"/>
+      <c r="I127" s="3" t="inlineStr"/>
+      <c r="J127" s="3" t="inlineStr"/>
+      <c r="K127" s="3" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L127" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M127" s="3" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>90481565100016</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>SAS EFB WALLONS</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>6 rue des Wallons</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>75013</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr"/>
+      <c r="I128" s="2" t="inlineStr"/>
+      <c r="J128" s="2" t="inlineStr"/>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L128" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M128" s="2" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>82206536300035</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>PAN-PAN</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>121 RUE DE LA ROQUETTE</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H129" s="3" t="inlineStr"/>
+      <c r="I129" s="3" t="inlineStr"/>
+      <c r="J129" s="3" t="inlineStr"/>
+      <c r="K129" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L129" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M129" s="3" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>79867433900014</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>BOULANGERIE BEN MASSAOUD</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>17 rue d Aligre</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>75012</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr"/>
+      <c r="I130" s="2" t="inlineStr"/>
+      <c r="J130" s="2" t="inlineStr"/>
+      <c r="K130" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L130" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M130" s="2" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>88119630700022</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>LES DELICES DE TUNIS</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>47 boulevard de Belleville</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="G131" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H131" s="3" t="inlineStr"/>
+      <c r="I131" s="3" t="inlineStr"/>
+      <c r="J131" s="3" t="inlineStr"/>
+      <c r="K131" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L131" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M131" s="3" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>88793457800014</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>LES 4 PETITS PAINS HELALI</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>114 boulevard de la Villette</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>75019</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr"/>
+      <c r="I132" s="2" t="inlineStr"/>
+      <c r="J132" s="2" t="inlineStr"/>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L132" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M132" s="2" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>81388063000013</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>BOULANGERIE PATISSERIE OUNISSI</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>138 Rue du Faubourg Saint-Antoine</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>75012</t>
+        </is>
+      </c>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="H133" s="3" t="inlineStr"/>
+      <c r="I133" s="3" t="inlineStr"/>
+      <c r="J133" s="3" t="inlineStr"/>
+      <c r="K133" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L133" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M133" s="3" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>82203977200022</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>BELALO</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>8 RUE DE BELLEVILLE</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>75020</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>0142237824</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr"/>
+      <c r="J134" s="2" t="inlineStr"/>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L134" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M134" s="2" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>40886430400014</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>AUGUSTIN SD 28</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr">
+        <is>
+          <t>28 rue DE LA PEPINIERE</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="G135" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H135" s="3" t="inlineStr">
+        <is>
+          <t>0144700410</t>
+        </is>
+      </c>
+      <c r="I135" s="3" t="inlineStr"/>
+      <c r="J135" s="3" t="inlineStr"/>
+      <c r="K135" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L135" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M135" s="3" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>89259933300010</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>LA COURONNE D'OR</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>78 boulevard de Belleville</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>75020</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr"/>
+      <c r="I136" s="2" t="inlineStr"/>
+      <c r="J136" s="2" t="inlineStr"/>
+      <c r="K136" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L136" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M136" s="2" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>55208329702404</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
+        <is>
+          <t>54 BOULEVARD DE L HOPITAL</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>75013</t>
+        </is>
+      </c>
+      <c r="G137" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H137" s="3" t="inlineStr"/>
+      <c r="I137" s="3" t="inlineStr"/>
+      <c r="J137" s="3" t="inlineStr"/>
+      <c r="K137" s="3" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L137" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M137" s="3" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>35352065300018</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>SOCIETE ORTEAUX</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>13B place d Aligre</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>75012</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr"/>
+      <c r="I138" s="2" t="inlineStr"/>
+      <c r="J138" s="2" t="inlineStr"/>
+      <c r="K138" s="2" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M138" s="2" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>52305151400017</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>MARCHE DELAMBRE</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>29 RUE DELAMBRE</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr">
+        <is>
+          <t>75014</t>
+        </is>
+      </c>
+      <c r="G139" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H139" s="3" t="inlineStr"/>
+      <c r="I139" s="3" t="inlineStr"/>
+      <c r="J139" s="3" t="inlineStr"/>
+      <c r="K139" s="3" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L139" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M139" s="3" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>82303638900018</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>MAISON R&amp;S LIEGE</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>58 RUE D AMSTERDAM</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr"/>
+      <c r="I140" s="2" t="inlineStr"/>
+      <c r="J140" s="2" t="inlineStr"/>
+      <c r="K140" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M140" s="2" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>85035251900019</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>BOULANGERIE BEN YEDDER</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
+        <is>
+          <t>4 RUE DE CLIGNANCOURT</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="inlineStr">
+        <is>
+          <t>75018</t>
+        </is>
+      </c>
+      <c r="G141" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H141" s="3" t="inlineStr"/>
+      <c r="I141" s="3" t="inlineStr"/>
+      <c r="J141" s="3" t="inlineStr"/>
+      <c r="K141" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L141" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M141" s="3" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>43247303100024</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>AMARBEN</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>28 RUE DU ROCHER</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>0148081272</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr"/>
+      <c r="J142" s="2" t="inlineStr"/>
+      <c r="K142" s="2" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M142" s="2" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C143" s="3" t="inlineStr">
+        <is>
+          <t>89511528500010</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>CHALA DISTRIBUTION</t>
+        </is>
+      </c>
+      <c r="E143" s="3" t="inlineStr">
+        <is>
+          <t>62 rue d Amsterdam</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr">
+        <is>
+          <t>75009</t>
+        </is>
+      </c>
+      <c r="G143" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H143" s="3" t="inlineStr"/>
+      <c r="I143" s="3" t="inlineStr"/>
+      <c r="J143" s="3" t="inlineStr"/>
+      <c r="K143" s="3" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L143" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M143" s="3" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>83496243300019</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>RACHA DISTRIBUTION</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>175 Rue du Faubourg Saint-Antoine</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr"/>
+      <c r="I144" s="2" t="inlineStr"/>
+      <c r="J144" s="2" t="inlineStr"/>
+      <c r="K144" s="2" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M144" s="2" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>81126116300018</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>SUPER STORE</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>19 RUE DE BELLEVILLE</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>75019</t>
+        </is>
+      </c>
+      <c r="G145" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H145" s="3" t="inlineStr"/>
+      <c r="I145" s="3" t="inlineStr"/>
+      <c r="J145" s="3" t="inlineStr"/>
+      <c r="K145" s="3" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L145" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M145" s="3" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>79871028100014</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>CHEMIN VERT DIS</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>127 RUE DU CHEMIN VERT</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr"/>
+      <c r="I146" s="2" t="inlineStr"/>
+      <c r="J146" s="2" t="inlineStr"/>
+      <c r="K146" s="2" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L146" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M146" s="2" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>91950833300011</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>BOULANGERIE OURIDA</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>32 rue de Belleville</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>75020</t>
+        </is>
+      </c>
+      <c r="G147" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H147" s="3" t="inlineStr"/>
+      <c r="I147" s="3" t="inlineStr"/>
+      <c r="J147" s="3" t="inlineStr"/>
+      <c r="K147" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L147" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M147" s="3" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>52990192800018</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>OUNISSI ABDELKARIM</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>132 RUE DU CHEMIN VERT</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr"/>
+      <c r="I148" s="2" t="inlineStr"/>
+      <c r="J148" s="2" t="inlineStr"/>
+      <c r="K148" s="2" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L148" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M148" s="2" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>82199589100024</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>LA ROYALE</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>45 RUE CROZATIER</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>75012</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H149" s="3" t="inlineStr"/>
+      <c r="I149" s="3" t="inlineStr"/>
+      <c r="J149" s="3" t="inlineStr"/>
+      <c r="K149" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L149" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M149" s="3" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>83085601900021</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>ANASANA</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>13 RUE ETIENNE DOLET</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>75020</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr"/>
+      <c r="I150" s="2" t="inlineStr"/>
+      <c r="J150" s="2" t="inlineStr"/>
+      <c r="K150" s="2" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L150" s="2" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M150" s="2" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>81740350400019</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>HOLDING BOULANGERIE</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>51 rue de Laborde</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H151" s="3" t="inlineStr"/>
+      <c r="I151" s="3" t="inlineStr"/>
+      <c r="J151" s="3" t="inlineStr"/>
+      <c r="K151" s="3" t="inlineStr">
+        <is>
+          <t>1071C</t>
+        </is>
+      </c>
+      <c r="L151" s="3" t="inlineStr">
+        <is>
+          <t>D1102</t>
+        </is>
+      </c>
+      <c r="M151" s="3" t="inlineStr"/>
+    </row>
+    <row r="152"/>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
         <is>
           <t>Total entreprises</t>
         </is>
       </c>
-      <c r="B103" s="4" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="4" t="inlineStr">
+      <c r="B153" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="4" t="inlineStr">
         <is>
           <t>dont LBB</t>
         </is>
       </c>
-      <c r="B104" s="4" t="n">
+      <c r="B154" s="4" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="4" t="inlineStr">
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
         <is>
           <t>dont LBA</t>
         </is>
       </c>
-      <c r="B105" s="4" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="4" t="inlineStr">
+      <c r="B155" s="4" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="4" t="inlineStr">
         <is>
           <t>dont LBB+LBA</t>
         </is>
       </c>
-      <c r="B106" s="4" t="n">
+      <c r="B156" s="4" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="4" t="inlineStr">
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
         <is>
           <t>Offre active</t>
         </is>
       </c>
-      <c r="B107" s="4" t="n">
+      <c r="B157" s="4" t="n">
         <v>17</v>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="4" t="inlineStr">
-        <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="B108" s="4" t="n">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="4" t="inlineStr">
+    <row r="158">
+      <c r="A158" s="4" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="n">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
         <is>
           <t>Sans téléphone</t>
         </is>
       </c>
-      <c r="B109" s="4" t="n">
-        <v>75</v>
+      <c r="B159" s="4" t="n">
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert Excel to clean state (remove incorrect phone data)
Phone enrichment via societe.com extracted the site's own service numbers
(0886311569, 0887316569) instead of real company phones — all major FR
directories block scraping or hide numbers behind JavaScript.

https://claude.ai/code/session_01XzkQisFxLhzSw3n843fcRb
</commit_message>
<xml_diff>
--- a/entreprises_alternance_paris.xlsx
+++ b/entreprises_alternance_paris.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Résultats_Scrap" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Résultats_Scrap" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
chore: update Excel output after LBB fix (62 contacts, 8 LBB+LBA)
https://claude.ai/code/session_01XzkQisFxLhzSw3n843fcRb
</commit_message>
<xml_diff>
--- a/entreprises_alternance_paris.xlsx
+++ b/entreprises_alternance_paris.xlsx
@@ -537,7 +537,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>LBB + LBA</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -547,39 +547,39 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>90353076400013</t>
+          <t>81012935300035</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TRAINING COMPETENCES</t>
+          <t>LE PAIN RETROUVE</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2 RUE CATULLE MENDES</t>
+          <t>18 RUE DES MARTYRS</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>75017</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>0749123569</t>
+          <t>0753210804</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>10.71C</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -592,7 +592,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>LBB + LBA</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -602,39 +602,39 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>97899031500019</t>
+          <t>40174230900024</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>L'EQUILIBRE</t>
+          <t>BOULANGERIE DE SEVRES</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>108 RUE BLOMET</t>
+          <t>54 RUE DE SEVRES</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>75015</t>
+          <t>75007</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>0148423046</t>
+          <t>0147833040</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr"/>
       <c r="J3" s="3" t="inlineStr"/>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>10.71C</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
@@ -647,7 +647,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>LBB + LBA</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -657,39 +657,39 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>80500000700031</t>
+          <t>50843100400037</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>LA MADELAINE 91 100</t>
+          <t>DE BELLES MANIERES</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>408 AVENUE JEAN JAURES</t>
+          <t>5 RUE DE TURBIGO</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>77190</t>
+          <t>75001</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>DAMMARIE-LES-LYS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>0665569709</t>
+          <t>0144829271</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>10.71C</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -702,54 +702,54 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>LBB + LBA</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
+          <t>Offre active</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>50843100400037</t>
+          <t>55208329701398</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>DE BELLES MANIERES</t>
+          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>5 RUE DE TURBIGO</t>
+          <t>54 AVENUE DU GENERAL LECLERC</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>75001</t>
+          <t>75014</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>0144829271</t>
+          <t>0145412698</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr"/>
       <c r="J5" s="3" t="inlineStr"/>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711E</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1103</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr"/>
@@ -757,54 +757,54 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>LBB + LBA</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
+          <t>Offre active</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>55203123900015</t>
+          <t>59202047300019</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>SOCIETE BOULANGERIE SAINT SAUVEUR COLLET</t>
+          <t>BOUCHERIE DEJEAN</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>100 RUE MONTORGUEIL</t>
+          <t>8 RUE DEJEAN</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>75002</t>
+          <t>75018</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>0145080006</t>
+          <t>0142527476</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4722Z</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1103</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr"/>
@@ -812,54 +812,54 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>LBB + LBA</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
+          <t>Offre active</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>79768080800012</t>
+          <t>41801191200015</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>SHAYNADIS</t>
+          <t>BOUCHERIE FAMILIALE III</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>53 RUE DE TURBIGO</t>
+          <t>23 RUE POULET</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75018</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>0144788040</t>
+          <t>0142629926</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr"/>
       <c r="J7" s="3" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>4722Z</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1103</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr"/>
@@ -867,54 +867,54 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>LBB + LBA</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
+          <t>Offre active</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>83218519300014</t>
+          <t>55208329700192</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>ABKH BOULANGERIE</t>
+          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>351 RUE SAINT MARTIN</t>
+          <t>52 RUE PIERRE FONTAINE</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>0656740881</t>
+          <t>0145269383</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711E</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1103</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr"/>
@@ -922,54 +922,54 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>LBB + LBA</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
+          <t>Offre active</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>91514335800017</t>
+          <t>54210134000017</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>LT2G</t>
+          <t>SOC ROBERT ET RENE</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>183 RUE DU TEMPLE</t>
+          <t>13 Rue du Faubourg du Temple</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>0134697793</t>
+          <t>0142082284</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr"/>
       <c r="J9" s="3" t="inlineStr"/>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4722Z</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1103</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr"/>
@@ -982,27 +982,27 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
+          <t>Offre active</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>32930252500020</t>
+          <t>90353076400013</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>MAISON MULOT SAS</t>
+          <t>TRAINING COMPETENCES</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>76 RUE DE SEINE</t>
+          <t>2 RUE CATULLE MENDES</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>75017</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1012,14 +1012,14 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>0143268577</t>
+          <t>0749123569</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1037,27 +1037,27 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
+          <t>Offre active</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>84166072300013</t>
+          <t>97899031500019</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>LP PROD</t>
+          <t>L'EQUILIBRE</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>12 rue du faubourg Poissonniere</t>
+          <t>108 RUE BLOMET</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75015</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -1067,14 +1067,14 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>0142385509</t>
+          <t>0148423046</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr"/>
       <c r="J11" s="3" t="inlineStr"/>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
@@ -1092,44 +1092,44 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
+          <t>Offre active</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>90162631700019</t>
+          <t>80500000700031</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>MAISON ISLAND</t>
+          <t>LA MADELAINE 91 100</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>8 rue des Filles du Calvaire</t>
+          <t>408 AVENUE JEAN JAURES</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>77190</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>DAMMARIE-LES-LYS</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>0647915566</t>
+          <t>0665569709</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1152,22 +1152,22 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>45045418600013</t>
+          <t>55203123900015</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>COFIGILLES</t>
+          <t>SOCIETE BOULANGERIE SAINT SAUVEUR COLLET</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>24 RUE SAINT GILLES</t>
+          <t>100 RUE MONTORGUEIL</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75002</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1177,14 +1177,14 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>0967452096</t>
+          <t>0145080006</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr"/>
       <c r="J13" s="3" t="inlineStr"/>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -1207,22 +1207,22 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>55208329701430</t>
+          <t>79768080800012</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
+          <t>SHAYNADIS</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>7 RUE DU DRAGON</t>
+          <t>53 RUE DE TURBIGO</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>0145481808</t>
+          <t>0144788040</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1262,22 +1262,22 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>75198013700028</t>
+          <t>83218519300014</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>TAL</t>
+          <t>ABKH BOULANGERIE</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>29 RUE SAINT ANTOINE</t>
+          <t>351 RUE SAINT MARTIN</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>75004</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>0235489596</t>
+          <t>0656740881</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr"/>
@@ -1317,22 +1317,22 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>33496216400011</t>
+          <t>91514335800017</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>SOGIBERGERE</t>
+          <t>LT2G</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>5 RUE GEOFFROY MARIE</t>
+          <t>183 RUE DU TEMPLE</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1342,14 +1342,14 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>0142463633</t>
+          <t>0134697793</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1372,22 +1372,22 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>52022307400037</t>
+          <t>32930252500020</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>LE PETIT MITRON</t>
+          <t>MAISON MULOT SAS</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>8 rue Oberkampf</t>
+          <t>76 RUE DE SEINE</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>0145411655</t>
+          <t>0143268577</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr"/>
@@ -1427,22 +1427,22 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>80403394200017</t>
+          <t>84166072300013</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>LES DELICES DE LAFAYETTE</t>
+          <t>LP PROD</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>1 rue de Provence</t>
+          <t>12 rue du faubourg Poissonniere</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1452,7 +1452,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>0153340875</t>
+          <t>0142385509</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -1482,22 +1482,22 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>80302565900019</t>
+          <t>90162631700019</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>LE TEMPS DU REVE</t>
+          <t>MAISON ISLAND</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>20 RUE JEAN PIERRE TIMBAUD</t>
+          <t>8 rue des Filles du Calvaire</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1507,7 +1507,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>0982507448</t>
+          <t>0647915566</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr"/>
@@ -1537,22 +1537,22 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>79124664800012</t>
+          <t>45045418600013</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>SARL RENNES 81</t>
+          <t>COFIGILLES</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>81 RUE DE RENNES</t>
+          <t>24 RUE SAINT GILLES</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1562,14 +1562,14 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>0620474041</t>
+          <t>0967452096</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1592,22 +1592,22 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>81012935300035</t>
+          <t>55208329701430</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>LE PAIN RETROUVE</t>
+          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>18 RUE DES MARTYRS</t>
+          <t>7 RUE DU DRAGON</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
@@ -1617,14 +1617,14 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>0753210804</t>
+          <t>0145481808</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr"/>
       <c r="J21" s="3" t="inlineStr"/>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
@@ -1647,22 +1647,22 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>53159116200015</t>
+          <t>75198013700028</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>LES DELICES DES FAUBOURGS</t>
+          <t>TAL</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>156 DU FAUBOURG SAINT MARTIN</t>
+          <t>29 RUE SAINT ANTOINE</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75004</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>0698011212</t>
+          <t>0235489596</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
@@ -1702,17 +1702,17 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>55208329701588</t>
+          <t>33496216400011</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
+          <t>SOGIBERGERE</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>52 RUE DE CAUMARTIN</t>
+          <t>5 RUE GEOFFROY MARIE</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>0144537979</t>
+          <t>0142463633</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr"/>
@@ -1757,17 +1757,17 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>84186128900012</t>
+          <t>52022307400037</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>ATELIER GUINOT BAKER</t>
+          <t>LE PETIT MITRON</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>6 RUE SAINT AMBROISE</t>
+          <t>8 rue Oberkampf</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>0662415274</t>
+          <t>0145411655</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
@@ -1812,22 +1812,22 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>53881702400010</t>
+          <t>80403394200017</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>HOUIRES TAHAR</t>
+          <t>LES DELICES DE LAFAYETTE</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>215 RUE SAINT MAUR</t>
+          <t>1 rue de Provence</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>0607463025</t>
+          <t>0153340875</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr"/>
@@ -1867,22 +1867,22 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>72205443400013</t>
+          <t>80302565900019</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>A LA BONNE SOURCE</t>
+          <t>LE TEMPS DU REVE</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>122 RUE MOUFFETARD</t>
+          <t>20 RUE JEAN PIERRE TIMBAUD</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1892,14 +1892,14 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>0143312963</t>
+          <t>0982507448</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -1922,22 +1922,22 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>83254766500014</t>
+          <t>79124664800012</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>SARL BRUMANO</t>
+          <t>SARL RENNES 81</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>83 RUE DE MAUBEUGE</t>
+          <t>81 RUE DE RENNES</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1947,7 +1947,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>0630321473</t>
+          <t>0620474041</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr"/>
@@ -1977,22 +1977,22 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>40174230900024</t>
+          <t>53159116200015</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>BOULANGERIE DE SEVRES</t>
+          <t>LES DELICES DES FAUBOURGS</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>54 RUE DE SEVRES</t>
+          <t>156 DU FAUBOURG SAINT MARTIN</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>75007</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>0147833040</t>
+          <t>0698011212</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -2032,22 +2032,22 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>80348700800028</t>
+          <t>55208329701588</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>SARLU AUX DELICES DE LOLO</t>
+          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>92 avenue de la Republique</t>
+          <t>52 RUE DE CAUMARTIN</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -2057,14 +2057,14 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>0148057385</t>
+          <t>0144537979</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr"/>
       <c r="J29" s="3" t="inlineStr"/>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
@@ -2087,22 +2087,22 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>35088924200011</t>
+          <t>84186128900012</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>SUPER DELAMBRE</t>
+          <t>ATELIER GUINOT BAKER</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>11 rue Delambre</t>
+          <t>6 RUE SAINT AMBROISE</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>75014</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2112,14 +2112,14 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>0142790787</t>
+          <t>0662415274</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -2142,32 +2142,32 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>82234103800013</t>
+          <t>53881702400010</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>BOULANGERIE SAINT ANTOINE</t>
+          <t>HOUIRES TAHAR</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>153 Rue du Faubourg Saint-Antoine</t>
+          <t>215 RUE SAINT MAUR</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>0143077758</t>
+          <t>0607463025</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr"/>
@@ -2197,22 +2197,22 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>88071932300029</t>
+          <t>72205443400013</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>LAUREDIS</t>
+          <t>A LA BONNE SOURCE</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>16B rue Pierre Fontaine</t>
+          <t>122 RUE MOUFFETARD</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>0611324848</t>
+          <t>0143312963</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -2252,22 +2252,22 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>82203977200022</t>
+          <t>83254766500014</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>BELALO</t>
+          <t>SARL BRUMANO</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>8 RUE DE BELLEVILLE</t>
+          <t>83 RUE DE MAUBEUGE</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>75020</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -2277,14 +2277,14 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>0142237824</t>
+          <t>0630321473</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr"/>
       <c r="J33" s="3" t="inlineStr"/>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
@@ -2307,22 +2307,22 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>40886430400014</t>
+          <t>80348700800028</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>AUGUSTIN SD 28</t>
+          <t>SARLU AUX DELICES DE LOLO</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>28 rue DE LA PEPINIERE</t>
+          <t>92 avenue de la Republique</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>75008</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>0144700410</t>
+          <t>0148057385</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
@@ -2362,22 +2362,22 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>43247303100024</t>
+          <t>35088924200011</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>AMARBEN</t>
+          <t>SUPER DELAMBRE</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>28 RUE DU ROCHER</t>
+          <t>11 rue Delambre</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>75008</t>
+          <t>75014</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -2387,7 +2387,7 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>0148081272</t>
+          <t>0142790787</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr"/>
@@ -2417,32 +2417,32 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>88887990500014</t>
+          <t>82234103800013</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>LIBERTE SAINT-DOMINIQUE</t>
+          <t>BOULANGERIE SAINT ANTOINE</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>58 rue Saint Dominique</t>
+          <t>153 Rue du Faubourg Saint-Antoine</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>75007</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>0659707911</t>
+          <t>0143077758</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -2472,22 +2472,22 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>41410339000020</t>
+          <t>88071932300029</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>SERVIDIS</t>
+          <t>LAUREDIS</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>14 rue Paul Bert</t>
+          <t>16B rue Pierre Fontaine</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G37" s="3" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>0143794343</t>
+          <t>0611324848</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr"/>
@@ -2527,22 +2527,22 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>83387608900016</t>
+          <t>82203977200022</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>BOULANGERIE O'SAINT HONORE</t>
+          <t>BELALO</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>97 RUE DU FBG ST HONORE</t>
+          <t>8 RUE DE BELLEVILLE</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>75008</t>
+          <t>75020</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2552,14 +2552,14 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>boulangerieosainthonore@gmail.com</t>
+          <t>0142237824</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -2582,22 +2582,22 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>38080133200020</t>
+          <t>40886430400014</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>PAIN POUJAURAN DIFFUSION</t>
+          <t>AUGUSTIN SD 28</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>18 RUE JEAN NICOT</t>
+          <t>28 rue DE LA PEPINIERE</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>75007</t>
+          <t>75008</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>0147058088</t>
+          <t>0144700410</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr"/>
@@ -2637,22 +2637,22 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>31667390400041</t>
+          <t>43247303100024</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>LE PETIT BOULE</t>
+          <t>AMARBEN</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>23B AVENUE DE LA MOTTE PICQUET</t>
+          <t>28 RUE DU ROCHER</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>75007</t>
+          <t>75008</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2662,14 +2662,14 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>0145517748</t>
+          <t>0148081272</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -2692,22 +2692,22 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>56206051700033</t>
+          <t>88887990500014</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>BOUCHERIE PARISIENNE DEBRAY</t>
+          <t>LIBERTE SAINT-DOMINIQUE</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>47T boulevard Saint Germain</t>
+          <t>58 rue Saint Dominique</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75007</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -2717,19 +2717,19 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>0143541122</t>
+          <t>0659707911</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr"/>
       <c r="J41" s="3" t="inlineStr"/>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr"/>
@@ -2747,22 +2747,22 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>53305173600015</t>
+          <t>41410339000020</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>DOYAJI</t>
+          <t>SERVIDIS</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>58 RUE SAINTE ANNE</t>
+          <t>14 rue Paul Bert</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>75002</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2772,19 +2772,19 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>0142966809</t>
+          <t>0143794343</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr"/>
@@ -2802,22 +2802,22 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>82362993600027</t>
+          <t>83387608900016</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>MEDIUM RARE</t>
+          <t>BOULANGERIE O'SAINT HONORE</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>7 rue Jean Pierre Timbaud</t>
+          <t>97 RUE DU FBG ST HONORE</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75008</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -2827,19 +2827,19 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>0146867550</t>
+          <t>boulangerieosainthonore@gmail.com</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr"/>
       <c r="J43" s="3" t="inlineStr"/>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>1011Z</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M43" s="3" t="inlineStr"/>
@@ -2857,44 +2857,44 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>54210134000017</t>
+          <t>38080133200020</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>SOC ROBERT ET RENE</t>
+          <t>PAIN POUJAURAN DIFFUSION</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>13 Rue du Faubourg du Temple</t>
+          <t>18 RUE JEAN NICOT</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75007</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>0142082284</t>
+          <t>0147058088</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr"/>
@@ -2912,22 +2912,22 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>79915248300027</t>
+          <t>31667390400041</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>LA BOUCHERIE DES FINS GOURMETS</t>
+          <t>LE PETIT BOULE</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>202 RUE SAINT JACQUES</t>
+          <t>23B AVENUE DE LA MOTTE PICQUET</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75007</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -2937,19 +2937,19 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>0139587749</t>
+          <t>0145517748</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr"/>
       <c r="J45" s="3" t="inlineStr"/>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr"/>
@@ -2967,22 +2967,22 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>37940157300017</t>
+          <t>56206051700033</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>BOUCHERIE OBERKAMPF</t>
+          <t>BOUCHERIE PARISIENNE DEBRAY</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>38 rue Oberkampf</t>
+          <t>47T boulevard Saint Germain</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>0147007409</t>
+          <t>0143541122</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr"/>
@@ -3022,22 +3022,22 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>84112278100013</t>
+          <t>53305173600015</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>MON LOUCHEBEM BIO</t>
+          <t>DOYAJI</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>85B BOULEVARD DE MAGENTA</t>
+          <t>58 RUE SAINTE ANNE</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75002</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>0634374149</t>
+          <t>0142966809</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr"/>
@@ -3077,39 +3077,39 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>44515584900018</t>
+          <t>82362993600027</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>DJUDJURA BLIDA</t>
+          <t>MEDIUM RARE</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>91 Rue du Faubourg du Temple</t>
+          <t>7 rue Jean Pierre Timbaud</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>0142085062</t>
+          <t>0146867550</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>1011Z</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
@@ -3132,22 +3132,22 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>42454439300020</t>
+          <t>79915248300027</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>DESPRES LUDOVIC</t>
+          <t>LA BOUCHERIE DES FINS GOURMETS</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>79 BOULEVARD SAINT MARCEL</t>
+          <t>202 RUE SAINT JACQUES</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>75013</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>0143315737</t>
+          <t>0139587749</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr"/>
@@ -3187,22 +3187,22 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>55208329700192</t>
+          <t>37940157300017</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
+          <t>BOUCHERIE OBERKAMPF</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>52 RUE PIERRE FONTAINE</t>
+          <t>38 rue Oberkampf</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -3212,14 +3212,14 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>0145269383</t>
+          <t>0147007409</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>4711E</t>
+          <t>4722Z</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
@@ -3242,22 +3242,22 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>50178435900017</t>
+          <t>84112278100013</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>T.B.S.</t>
+          <t>MON LOUCHEBEM BIO</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>106 RUE DE CHARONNE</t>
+          <t>85B BOULEVARD DE MAGENTA</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>0143709250</t>
+          <t>0634374149</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr"/>
@@ -3297,32 +3297,32 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>48336842900039</t>
+          <t>44515584900018</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>LE COUTEAU D ARGENT</t>
+          <t>DJUDJURA BLIDA</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>63 BOULEVARD MALESHERBES</t>
+          <t>91 Rue du Faubourg du Temple</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>75008</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>0156280990</t>
+          <t>0142085062</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
@@ -3352,22 +3352,22 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>59202047300019</t>
+          <t>42454439300020</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>BOUCHERIE DEJEAN</t>
+          <t>DESPRES LUDOVIC</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>8 RUE DEJEAN</t>
+          <t>79 BOULEVARD SAINT MARCEL</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>75018</t>
+          <t>75013</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -3377,7 +3377,7 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>0142527476</t>
+          <t>0143315737</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr"/>
@@ -3407,22 +3407,22 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>41801191200015</t>
+          <t>50178435900017</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>BOUCHERIE FAMILIALE III</t>
+          <t>T.B.S.</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>23 RUE POULET</t>
+          <t>106 RUE DE CHARONNE</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>75018</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>0142629926</t>
+          <t>0143709250</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr"/>
@@ -3462,22 +3462,22 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>53982691700020</t>
+          <t>48336842900039</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>BOUCHERIE DAGUERRE</t>
+          <t>LE COUTEAU D ARGENT</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>29 RUE DAGUERRE</t>
+          <t>63 BOULEVARD MALESHERBES</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>75014</t>
+          <t>75008</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>0143202478</t>
+          <t>0156280990</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr"/>
@@ -3517,22 +3517,22 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>52842513500068</t>
+          <t>53982691700020</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>NEDJAH DISTRIBUTION</t>
+          <t>BOUCHERIE DAGUERRE</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>385 RUE DES PYRENEES</t>
+          <t>29 RUE DAGUERRE</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>75020</t>
+          <t>75014</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -3542,14 +3542,14 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>0153241081</t>
+          <t>0143202478</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>4722Z</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
@@ -3572,22 +3572,22 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>55208329701604</t>
+          <t>52842513500068</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
+          <t>NEDJAH DISTRIBUTION</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>43 AVENUE DE CLICHY</t>
+          <t>385 RUE DES PYRENEES</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>75017</t>
+          <t>75020</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>0142932204</t>
+          <t>0153241081</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr"/>
@@ -3627,22 +3627,22 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>71203743100012</t>
+          <t>55208329701604</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>SUPER DOMINIQUE</t>
+          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>143 rue Saint Dominique</t>
+          <t>43 AVENUE DE CLICHY</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>75007</t>
+          <t>75017</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>0145514243</t>
+          <t>0142932204</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr"/>
@@ -3682,22 +3682,22 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>79295582500015</t>
+          <t>71203743100012</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>BOUCHERIE FAMILIALE RIQUET</t>
+          <t>SUPER DOMINIQUE</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>98 RUE RIQUET</t>
+          <t>143 rue Saint Dominique</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>75018</t>
+          <t>75007</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -3707,14 +3707,14 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>0142050025</t>
+          <t>0145514243</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr"/>
       <c r="J59" s="3" t="inlineStr"/>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
@@ -3737,17 +3737,17 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>80762479600015</t>
+          <t>79295582500015</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>NELIHAM</t>
+          <t>BOUCHERIE FAMILIALE RIQUET</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>136 RUE LAMARCK</t>
+          <t>98 RUE RIQUET</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -3762,14 +3762,14 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>0153313143</t>
+          <t>0142050025</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>4722Z</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
@@ -3792,22 +3792,22 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>55208329701398</t>
+          <t>80762479600015</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
+          <t>NELIHAM</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>54 AVENUE DU GENERAL LECLERC</t>
+          <t>136 RUE LAMARCK</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>75014</t>
+          <t>75018</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -3817,14 +3817,14 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>0145412698</t>
+          <t>0153313143</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr"/>
       <c r="J61" s="3" t="inlineStr"/>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>4711E</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L61" s="3" t="inlineStr">
@@ -3972,7 +3972,7 @@
         </is>
       </c>
       <c r="B67" s="4" t="n">
-        <v>62</v>
+        <v>54</v>
       </c>
     </row>
     <row r="68">
@@ -3982,7 +3982,7 @@
         </is>
       </c>
       <c r="B68" s="4" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="69">
@@ -3992,7 +3992,7 @@
         </is>
       </c>
       <c r="B69" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="70">
@@ -4002,7 +4002,7 @@
         </is>
       </c>
       <c r="B70" s="4" t="n">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="71">

</xml_diff>

<commit_message>
feat: ajouter source OFT (Offres d'emploi France Travail v2)
- Nouvelle source OFT via API api_offresdemploiv2 / o2dsoffre
- ROME D1102/D1103/D1104/D1101 sur 8 départements IDF
- Extrait contact.telephone des offres d'emploi actives
- Dédup OFT par (nom_entreprise, code_postal) + enrichissement SIRET
- Résultat : 74 contacts avec téléphone (+12 vs 62 avant)
- Synthèse : 54 LBA + 11 OFT + 9 multi-sources

https://claude.ai/code/session_01XzkQisFxLhzSw3n843fcRb
</commit_message>
<xml_diff>
--- a/entreprises_alternance_paris.xlsx
+++ b/entreprises_alternance_paris.xlsx
@@ -449,16 +449,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M71"/>
+  <dimension ref="A1:M84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="44" customWidth="1" min="4" max="4"/>
     <col width="37" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="37" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
@@ -1142,49 +1142,45 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>LBA + OFT</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
+          <t>Offre active</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>55203123900015</t>
+          <t>80350239200019</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>SOCIETE BOULANGERIE SAINT SAUVEUR COLLET</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>100 RUE MONTORGUEIL</t>
-        </is>
-      </c>
+          <t>L'ATELIER DES GOURMANDS</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>75002</t>
+          <t>93160</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Noisy-le-Grand</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>0145080006</t>
+          <t>0661914070</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr"/>
       <c r="J13" s="3" t="inlineStr"/>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
@@ -1197,54 +1193,46 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>OFT</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>79768080800012</t>
-        </is>
-      </c>
+          <t>Offre active</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>SHAYNADIS</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>53 RUE DE TURBIGO</t>
-        </is>
-      </c>
+          <t>Le grenier à pain</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>75015</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>0144788040</t>
+          <t>0673797642</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1104</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr"/>
@@ -1252,49 +1240,41 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>OFT</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>83218519300014</t>
-        </is>
-      </c>
+          <t>Offre active</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr"/>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>ABKH BOULANGERIE</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>351 RUE SAINT MARTIN</t>
-        </is>
-      </c>
+          <t>BOULANGERIE DE LA PLACE</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>77550</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Moissy Cramayel</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>0656740881</t>
+          <t>0651017305</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr"/>
       <c r="J15" s="3" t="inlineStr"/>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
@@ -1307,54 +1287,46 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>OFT</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>91514335800017</t>
-        </is>
-      </c>
+          <t>Offre active</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>LT2G</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>183 RUE DU TEMPLE</t>
-        </is>
-      </c>
+          <t>LES TOQUES DU PAIN</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>91590</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Baulne</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>0134697793</t>
+          <t>0768292517</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1104</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr"/>
@@ -1362,49 +1334,41 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>OFT</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>32930252500020</t>
-        </is>
-      </c>
+          <t>Offre active</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>MAISON MULOT SAS</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>76 RUE DE SEINE</t>
-        </is>
-      </c>
+          <t>LE PETIT REMY</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>92300</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Levallois Perret</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>0143268577</t>
+          <t>0682095143</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr"/>
       <c r="J17" s="3" t="inlineStr"/>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
@@ -1417,54 +1381,46 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>OFT</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>84166072300013</t>
-        </is>
-      </c>
+          <t>Offre active</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>LP PROD</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>12 rue du faubourg Poissonniere</t>
-        </is>
-      </c>
+          <t>Boucherie MODERNE</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>92110</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Clichy</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>0142385509</t>
+          <t>0662892486</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>47.22Z</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1101</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr"/>
@@ -1472,49 +1428,41 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>OFT</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>90162631700019</t>
-        </is>
-      </c>
+          <t>Offre active</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr"/>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>MAISON ISLAND</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>8 rue des Filles du Calvaire</t>
-        </is>
-      </c>
+          <t>AUX SAVEURS GOURMANDES</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>93140</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Bondy</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>0647915566</t>
+          <t>0626783291</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr"/>
       <c r="J19" s="3" t="inlineStr"/>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L19" s="3" t="inlineStr">
@@ -1527,49 +1475,41 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>OFT</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>45045418600013</t>
-        </is>
-      </c>
+          <t>Offre active</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>COFIGILLES</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>24 RUE SAINT GILLES</t>
-        </is>
-      </c>
+          <t>SAS LA TRADITION</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>75003</t>
+          <t>93140</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Bondy</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>0967452096</t>
+          <t>0601791213</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -1582,49 +1522,41 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>OFT</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>55208329701430</t>
-        </is>
-      </c>
+          <t>Offre active</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr"/>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>7 RUE DU DRAGON</t>
-        </is>
-      </c>
+          <t>BOULANGERIE CHOUQUETTE</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>94320</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Thiais</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>0145481808</t>
+          <t>0651852127</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr"/>
       <c r="J21" s="3" t="inlineStr"/>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L21" s="3" t="inlineStr">
@@ -1637,49 +1569,41 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>OFT</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>75198013700028</t>
-        </is>
-      </c>
+          <t>Offre active</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>TAL</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>29 RUE SAINT ANTOINE</t>
-        </is>
-      </c>
+          <t>LE FOURNIL DES CHAMPS</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>75004</t>
+          <t>95230</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Soisy Sous Montmorency</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>0235489596</t>
+          <t>0671801580</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -1692,54 +1616,46 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>OFT</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>33496216400011</t>
-        </is>
-      </c>
+          <t>Offre active</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr"/>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>SOGIBERGERE</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>5 RUE GEOFFROY MARIE</t>
-        </is>
-      </c>
+          <t>Mr rabineau</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>95580</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Andilly</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>0142463633</t>
+          <t>0614213953</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr"/>
       <c r="J23" s="3" t="inlineStr"/>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>94.11Z</t>
         </is>
       </c>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1104</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr"/>
@@ -1747,54 +1663,46 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>LBA</t>
+          <t>OFT</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>52022307400037</t>
-        </is>
-      </c>
+          <t>Offre active</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>LE PETIT MITRON</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>8 rue Oberkampf</t>
-        </is>
-      </c>
+          <t>LE MOULIN DU LAC</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>95880</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Enghien Les Bains</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>0145411655</t>
+          <t>0675074174</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>10.71C</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>D1102</t>
+          <t>D1104</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr"/>
@@ -1812,22 +1720,22 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>80403394200017</t>
+          <t>55203123900015</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>LES DELICES DE LAFAYETTE</t>
+          <t>SOCIETE BOULANGERIE SAINT SAUVEUR COLLET</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>1 rue de Provence</t>
+          <t>100 RUE MONTORGUEIL</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75002</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -1837,7 +1745,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>0153340875</t>
+          <t>0145080006</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr"/>
@@ -1867,22 +1775,22 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>80302565900019</t>
+          <t>79768080800012</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>LE TEMPS DU REVE</t>
+          <t>SHAYNADIS</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>20 RUE JEAN PIERRE TIMBAUD</t>
+          <t>53 RUE DE TURBIGO</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1892,14 +1800,14 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>0982507448</t>
+          <t>0144788040</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -1922,22 +1830,22 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>79124664800012</t>
+          <t>83218519300014</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>SARL RENNES 81</t>
+          <t>ABKH BOULANGERIE</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>81 RUE DE RENNES</t>
+          <t>351 RUE SAINT MARTIN</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>75006</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1947,7 +1855,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>0620474041</t>
+          <t>0656740881</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr"/>
@@ -1977,22 +1885,22 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>53159116200015</t>
+          <t>91514335800017</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>LES DELICES DES FAUBOURGS</t>
+          <t>LT2G</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>156 DU FAUBOURG SAINT MARTIN</t>
+          <t>183 RUE DU TEMPLE</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2002,7 +1910,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>0698011212</t>
+          <t>0134697793</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -2032,22 +1940,22 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>55208329701588</t>
+          <t>32930252500020</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
+          <t>MAISON MULOT SAS</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>52 RUE DE CAUMARTIN</t>
+          <t>76 RUE DE SEINE</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>75009</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -2057,14 +1965,14 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>0144537979</t>
+          <t>0143268577</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr"/>
       <c r="J29" s="3" t="inlineStr"/>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr">
@@ -2087,22 +1995,22 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>84186128900012</t>
+          <t>84166072300013</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>ATELIER GUINOT BAKER</t>
+          <t>LP PROD</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>6 RUE SAINT AMBROISE</t>
+          <t>12 rue du faubourg Poissonniere</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -2112,7 +2020,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>0662415274</t>
+          <t>0142385509</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -2142,22 +2050,22 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>53881702400010</t>
+          <t>90162631700019</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>HOUIRES TAHAR</t>
+          <t>MAISON ISLAND</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>215 RUE SAINT MAUR</t>
+          <t>8 rue des Filles du Calvaire</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -2167,7 +2075,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>0607463025</t>
+          <t>0647915566</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr"/>
@@ -2197,22 +2105,22 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>72205443400013</t>
+          <t>45045418600013</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>A LA BONNE SOURCE</t>
+          <t>COFIGILLES</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>122 RUE MOUFFETARD</t>
+          <t>24 RUE SAINT GILLES</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75003</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -2222,7 +2130,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>0143312963</t>
+          <t>0967452096</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
@@ -2252,22 +2160,22 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>83254766500014</t>
+          <t>55208329701430</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>SARL BRUMANO</t>
+          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>83 RUE DE MAUBEUGE</t>
+          <t>7 RUE DU DRAGON</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -2277,14 +2185,14 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>0630321473</t>
+          <t>0145481808</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr"/>
       <c r="J33" s="3" t="inlineStr"/>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L33" s="3" t="inlineStr">
@@ -2307,22 +2215,22 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>80348700800028</t>
+          <t>75198013700028</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>SARLU AUX DELICES DE LOLO</t>
+          <t>TAL</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>92 avenue de la Republique</t>
+          <t>29 RUE SAINT ANTOINE</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75004</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2332,7 +2240,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>0148057385</t>
+          <t>0235489596</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr"/>
@@ -2362,22 +2270,22 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>35088924200011</t>
+          <t>33496216400011</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>SUPER DELAMBRE</t>
+          <t>SOGIBERGERE</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>11 rue Delambre</t>
+          <t>5 RUE GEOFFROY MARIE</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>75014</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -2387,7 +2295,7 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>0142790787</t>
+          <t>0142463633</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr"/>
@@ -2417,17 +2325,17 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>82234103800013</t>
+          <t>52022307400037</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>BOULANGERIE SAINT ANTOINE</t>
+          <t>LE PETIT MITRON</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>153 Rue du Faubourg Saint-Antoine</t>
+          <t>8 rue Oberkampf</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2437,12 +2345,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>0143077758</t>
+          <t>0145411655</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr"/>
@@ -2472,17 +2380,17 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>88071932300029</t>
+          <t>80403394200017</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>LAUREDIS</t>
+          <t>LES DELICES DE LAFAYETTE</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>16B rue Pierre Fontaine</t>
+          <t>1 rue de Provence</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -2497,14 +2405,14 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>0611324848</t>
+          <t>0153340875</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr"/>
       <c r="J37" s="3" t="inlineStr"/>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L37" s="3" t="inlineStr">
@@ -2527,22 +2435,22 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>82203977200022</t>
+          <t>80302565900019</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>BELALO</t>
+          <t>LE TEMPS DU REVE</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>8 RUE DE BELLEVILLE</t>
+          <t>20 RUE JEAN PIERRE TIMBAUD</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>75020</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2552,14 +2460,14 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>0142237824</t>
+          <t>0982507448</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -2582,22 +2490,22 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>40886430400014</t>
+          <t>79124664800012</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>AUGUSTIN SD 28</t>
+          <t>SARL RENNES 81</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>28 rue DE LA PEPINIERE</t>
+          <t>81 RUE DE RENNES</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>75008</t>
+          <t>75006</t>
         </is>
       </c>
       <c r="G39" s="3" t="inlineStr">
@@ -2607,7 +2515,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>0144700410</t>
+          <t>0620474041</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr"/>
@@ -2637,22 +2545,22 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>43247303100024</t>
+          <t>53159116200015</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>AMARBEN</t>
+          <t>LES DELICES DES FAUBOURGS</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>28 RUE DU ROCHER</t>
+          <t>156 DU FAUBOURG SAINT MARTIN</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>75008</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2662,14 +2570,14 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>0148081272</t>
+          <t>0698011212</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -2692,22 +2600,22 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>88887990500014</t>
+          <t>55208329701588</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>LIBERTE SAINT-DOMINIQUE</t>
+          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>58 rue Saint Dominique</t>
+          <t>52 RUE DE CAUMARTIN</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>75007</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -2717,14 +2625,14 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>0659707911</t>
+          <t>0144537979</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr"/>
       <c r="J41" s="3" t="inlineStr"/>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L41" s="3" t="inlineStr">
@@ -2747,17 +2655,17 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>41410339000020</t>
+          <t>84186128900012</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>SERVIDIS</t>
+          <t>ATELIER GUINOT BAKER</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>14 rue Paul Bert</t>
+          <t>6 RUE SAINT AMBROISE</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -2772,14 +2680,14 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>0143794343</t>
+          <t>0662415274</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -2802,22 +2710,22 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>83387608900016</t>
+          <t>53881702400010</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>BOULANGERIE O'SAINT HONORE</t>
+          <t>HOUIRES TAHAR</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>97 RUE DU FBG ST HONORE</t>
+          <t>215 RUE SAINT MAUR</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>75008</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G43" s="3" t="inlineStr">
@@ -2827,7 +2735,7 @@
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
-          <t>boulangerieosainthonore@gmail.com</t>
+          <t>0607463025</t>
         </is>
       </c>
       <c r="I43" s="3" t="inlineStr"/>
@@ -2857,22 +2765,22 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>38080133200020</t>
+          <t>72205443400013</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>PAIN POUJAURAN DIFFUSION</t>
+          <t>A LA BONNE SOURCE</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>18 RUE JEAN NICOT</t>
+          <t>122 RUE MOUFFETARD</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>75007</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2882,14 +2790,14 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>0147058088</t>
+          <t>0143312963</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>1071C</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
@@ -2912,22 +2820,22 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>31667390400041</t>
+          <t>83254766500014</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>LE PETIT BOULE</t>
+          <t>SARL BRUMANO</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>23B AVENUE DE LA MOTTE PICQUET</t>
+          <t>83 RUE DE MAUBEUGE</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>75007</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -2937,7 +2845,7 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>0145517748</t>
+          <t>0630321473</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr"/>
@@ -2967,22 +2875,22 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>56206051700033</t>
+          <t>80348700800028</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>BOUCHERIE PARISIENNE DEBRAY</t>
+          <t>SARLU AUX DELICES DE LOLO</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>47T boulevard Saint Germain</t>
+          <t>92 avenue de la Republique</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -2992,19 +2900,19 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>0143541122</t>
+          <t>0148057385</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr"/>
@@ -3022,22 +2930,22 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>53305173600015</t>
+          <t>35088924200011</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>DOYAJI</t>
+          <t>SUPER DELAMBRE</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>58 RUE SAINTE ANNE</t>
+          <t>11 rue Delambre</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>75002</t>
+          <t>75014</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -3047,19 +2955,19 @@
       </c>
       <c r="H47" s="3" t="inlineStr">
         <is>
-          <t>0142966809</t>
+          <t>0142790787</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr"/>
       <c r="J47" s="3" t="inlineStr"/>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr"/>
@@ -3077,17 +2985,17 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>82362993600027</t>
+          <t>82234103800013</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM RARE</t>
+          <t>BOULANGERIE SAINT ANTOINE</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>7 rue Jean Pierre Timbaud</t>
+          <t>153 Rue du Faubourg Saint-Antoine</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3097,24 +3005,24 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>PARIS</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>0146867550</t>
+          <t>0143077758</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>1011Z</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr"/>
@@ -3132,22 +3040,22 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>79915248300027</t>
+          <t>88071932300029</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>LA BOUCHERIE DES FINS GOURMETS</t>
+          <t>LAUREDIS</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>202 RUE SAINT JACQUES</t>
+          <t>16B rue Pierre Fontaine</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>75005</t>
+          <t>75009</t>
         </is>
       </c>
       <c r="G49" s="3" t="inlineStr">
@@ -3157,19 +3065,19 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>0139587749</t>
+          <t>0611324848</t>
         </is>
       </c>
       <c r="I49" s="3" t="inlineStr"/>
       <c r="J49" s="3" t="inlineStr"/>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr"/>
@@ -3187,22 +3095,22 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>37940157300017</t>
+          <t>82203977200022</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>BOUCHERIE OBERKAMPF</t>
+          <t>BELALO</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>38 rue Oberkampf</t>
+          <t>8 RUE DE BELLEVILLE</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>75011</t>
+          <t>75020</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -3212,19 +3120,19 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>0147007409</t>
+          <t>0142237824</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr"/>
@@ -3242,22 +3150,22 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>84112278100013</t>
+          <t>40886430400014</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>MON LOUCHEBEM BIO</t>
+          <t>AUGUSTIN SD 28</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>85B BOULEVARD DE MAGENTA</t>
+          <t>28 rue DE LA PEPINIERE</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75008</t>
         </is>
       </c>
       <c r="G51" s="3" t="inlineStr">
@@ -3267,19 +3175,19 @@
       </c>
       <c r="H51" s="3" t="inlineStr">
         <is>
-          <t>0634374149</t>
+          <t>0144700410</t>
         </is>
       </c>
       <c r="I51" s="3" t="inlineStr"/>
       <c r="J51" s="3" t="inlineStr"/>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L51" s="3" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M51" s="3" t="inlineStr"/>
@@ -3297,44 +3205,44 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>44515584900018</t>
+          <t>43247303100024</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>DJUDJURA BLIDA</t>
+          <t>AMARBEN</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>91 Rue du Faubourg du Temple</t>
+          <t>28 RUE DU ROCHER</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>75010</t>
+          <t>75008</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>PARIS</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>0142085062</t>
+          <t>0148081272</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr"/>
@@ -3352,22 +3260,22 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>42454439300020</t>
+          <t>88887990500014</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>DESPRES LUDOVIC</t>
+          <t>LIBERTE SAINT-DOMINIQUE</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>79 BOULEVARD SAINT MARCEL</t>
+          <t>58 rue Saint Dominique</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>75013</t>
+          <t>75007</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
@@ -3377,19 +3285,19 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>0143315737</t>
+          <t>0659707911</t>
         </is>
       </c>
       <c r="I53" s="3" t="inlineStr"/>
       <c r="J53" s="3" t="inlineStr"/>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L53" s="3" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M53" s="3" t="inlineStr"/>
@@ -3407,17 +3315,17 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>50178435900017</t>
+          <t>41410339000020</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>T.B.S.</t>
+          <t>SERVIDIS</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>106 RUE DE CHARONNE</t>
+          <t>14 rue Paul Bert</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -3432,19 +3340,19 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>0143709250</t>
+          <t>0143794343</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>4711D</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr"/>
@@ -3462,17 +3370,17 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>48336842900039</t>
+          <t>83387608900016</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>LE COUTEAU D ARGENT</t>
+          <t>BOULANGERIE O'SAINT HONORE</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>63 BOULEVARD MALESHERBES</t>
+          <t>97 RUE DU FBG ST HONORE</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
@@ -3487,19 +3395,19 @@
       </c>
       <c r="H55" s="3" t="inlineStr">
         <is>
-          <t>0156280990</t>
+          <t>boulangerieosainthonore@gmail.com</t>
         </is>
       </c>
       <c r="I55" s="3" t="inlineStr"/>
       <c r="J55" s="3" t="inlineStr"/>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L55" s="3" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M55" s="3" t="inlineStr"/>
@@ -3517,22 +3425,22 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>53982691700020</t>
+          <t>38080133200020</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>BOUCHERIE DAGUERRE</t>
+          <t>PAIN POUJAURAN DIFFUSION</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>29 RUE DAGUERRE</t>
+          <t>18 RUE JEAN NICOT</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>75014</t>
+          <t>75007</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -3542,19 +3450,19 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>0143202478</t>
+          <t>0147058088</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr"/>
@@ -3572,22 +3480,22 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>52842513500068</t>
+          <t>31667390400041</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>NEDJAH DISTRIBUTION</t>
+          <t>LE PETIT BOULE</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>385 RUE DES PYRENEES</t>
+          <t>23B AVENUE DE LA MOTTE PICQUET</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>75020</t>
+          <t>75007</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
@@ -3597,19 +3505,19 @@
       </c>
       <c r="H57" s="3" t="inlineStr">
         <is>
-          <t>0153241081</t>
+          <t>0145517748</t>
         </is>
       </c>
       <c r="I57" s="3" t="inlineStr"/>
       <c r="J57" s="3" t="inlineStr"/>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>1071C</t>
         </is>
       </c>
       <c r="L57" s="3" t="inlineStr">
         <is>
-          <t>D1103</t>
+          <t>D1102</t>
         </is>
       </c>
       <c r="M57" s="3" t="inlineStr"/>
@@ -3627,22 +3535,22 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>55208329701604</t>
+          <t>56206051700033</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
+          <t>BOUCHERIE PARISIENNE DEBRAY</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>43 AVENUE DE CLICHY</t>
+          <t>47T boulevard Saint Germain</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>75017</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -3652,14 +3560,14 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>0142932204</t>
+          <t>0143541122</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="2" t="inlineStr"/>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>4722Z</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
@@ -3682,22 +3590,22 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>71203743100012</t>
+          <t>53305173600015</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>SUPER DOMINIQUE</t>
+          <t>DOYAJI</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>143 rue Saint Dominique</t>
+          <t>58 RUE SAINTE ANNE</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>75007</t>
+          <t>75002</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -3707,14 +3615,14 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>0145514243</t>
+          <t>0142966809</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr"/>
       <c r="J59" s="3" t="inlineStr"/>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>4722Z</t>
         </is>
       </c>
       <c r="L59" s="3" t="inlineStr">
@@ -3737,22 +3645,22 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>79295582500015</t>
+          <t>82362993600027</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>BOUCHERIE FAMILIALE RIQUET</t>
+          <t>MEDIUM RARE</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>98 RUE RIQUET</t>
+          <t>7 rue Jean Pierre Timbaud</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>75018</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -3762,14 +3670,14 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>0142050025</t>
+          <t>0146867550</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>4722Z</t>
+          <t>1011Z</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
@@ -3792,22 +3700,22 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>80762479600015</t>
+          <t>79915248300027</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>NELIHAM</t>
+          <t>LA BOUCHERIE DES FINS GOURMETS</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>136 RUE LAMARCK</t>
+          <t>202 RUE SAINT JACQUES</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>75018</t>
+          <t>75005</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -3817,14 +3725,14 @@
       </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
-          <t>0153313143</t>
+          <t>0139587749</t>
         </is>
       </c>
       <c r="I61" s="3" t="inlineStr"/>
       <c r="J61" s="3" t="inlineStr"/>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>4722Z</t>
         </is>
       </c>
       <c r="L61" s="3" t="inlineStr">
@@ -3847,22 +3755,22 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>32862092700017</t>
+          <t>37940157300017</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>SOCIETE DE DISTRIBUTION DUPLEIX SODIPLEI</t>
+          <t>BOUCHERIE OBERKAMPF</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>4 RUE DUPLEIX</t>
+          <t>38 rue Oberkampf</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>75015</t>
+          <t>75011</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -3872,14 +3780,14 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>0147343123</t>
+          <t>0147007409</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>4711D</t>
+          <t>4722Z</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
@@ -3902,22 +3810,22 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>41488533500037</t>
+          <t>84112278100013</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>BENSON</t>
+          <t>MON LOUCHEBEM BIO</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>121 rue de La Glaciere</t>
+          <t>85B BOULEVARD DE MAGENTA</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>75013</t>
+          <t>75010</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
@@ -3927,91 +3835,761 @@
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
-          <t>0153800805</t>
+          <t>0634374149</t>
         </is>
       </c>
       <c r="I63" s="3" t="inlineStr"/>
       <c r="J63" s="3" t="inlineStr"/>
       <c r="K63" s="3" t="inlineStr">
         <is>
+          <t>4722Z</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>44515584900018</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>DJUDJURA BLIDA</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>91 Rue du Faubourg du Temple</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>75010</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>0142085062</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>4722Z</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>42454439300020</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>DESPRES LUDOVIC</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>79 BOULEVARD SAINT MARCEL</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>75013</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>0143315737</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr"/>
+      <c r="J65" s="3" t="inlineStr"/>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>4722Z</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>50178435900017</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>T.B.S.</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>106 RUE DE CHARONNE</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>75011</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>0143709250</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>4722Z</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>48336842900039</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>LE COUTEAU D ARGENT</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>63 BOULEVARD MALESHERBES</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>75008</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>0156280990</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr"/>
+      <c r="J67" s="3" t="inlineStr"/>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>4722Z</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>53982691700020</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>BOUCHERIE DAGUERRE</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>29 RUE DAGUERRE</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>75014</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>0143202478</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>4722Z</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>52842513500068</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>NEDJAH DISTRIBUTION</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>385 RUE DES PYRENEES</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>75020</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>0153241081</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr"/>
+      <c r="J69" s="3" t="inlineStr"/>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
           <t>4711D</t>
         </is>
       </c>
-      <c r="L63" s="3" t="inlineStr">
+      <c r="L69" s="3" t="inlineStr">
         <is>
           <t>D1103</t>
         </is>
       </c>
-      <c r="M63" s="3" t="inlineStr"/>
-    </row>
-    <row r="64"/>
-    <row r="65">
-      <c r="A65" s="4" t="inlineStr">
+      <c r="M69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>55208329701604</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>MONOPRIX EXPLOITATION, PAR ABREVIATION M</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>43 AVENUE DE CLICHY</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>75017</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>0142932204</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>71203743100012</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>SUPER DOMINIQUE</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>143 rue Saint Dominique</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>75007</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>0145514243</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr"/>
+      <c r="J71" s="3" t="inlineStr"/>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M71" s="3" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>79295582500015</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>BOUCHERIE FAMILIALE RIQUET</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>98 RUE RIQUET</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>75018</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>0142050025</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>4722Z</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>80762479600015</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>NELIHAM</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>136 RUE LAMARCK</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>75018</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>0153313143</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr"/>
+      <c r="J73" s="3" t="inlineStr"/>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L73" s="3" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M73" s="3" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>32862092700017</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>SOCIETE DE DISTRIBUTION DUPLEIX SODIPLEI</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>4 RUE DUPLEIX</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>75015</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>0147343123</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>LBA</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>41488533500037</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>BENSON</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>121 rue de La Glaciere</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>75013</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>PARIS</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>0153800805</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr"/>
+      <c r="J75" s="3" t="inlineStr"/>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>4711D</t>
+        </is>
+      </c>
+      <c r="L75" s="3" t="inlineStr">
+        <is>
+          <t>D1103</t>
+        </is>
+      </c>
+      <c r="M75" s="3" t="inlineStr"/>
+    </row>
+    <row r="76"/>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
         <is>
           <t>Total entreprises</t>
         </is>
       </c>
-      <c r="B65" s="4" t="n">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="4" t="inlineStr">
+      <c r="B77" s="4" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
         <is>
           <t>dont LBB</t>
         </is>
       </c>
-      <c r="B66" s="4" t="n">
+      <c r="B78" s="4" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="4" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
         <is>
           <t>dont LBA</t>
         </is>
       </c>
-      <c r="B67" s="4" t="n">
+      <c r="B79" s="4" t="n">
         <v>54</v>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>dont LBB+LBA</t>
-        </is>
-      </c>
-      <c r="B68" s="4" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>dont OFT</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>dont multi-sources</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
         <is>
           <t>Offre active</t>
         </is>
       </c>
-      <c r="B69" s="4" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>Entreprise cible</t>
-        </is>
-      </c>
-      <c r="B70" s="4" t="n">
+      <c r="B82" s="4" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>Entreprise cible</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="n">
         <v>51</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
         <is>
           <t>Sans téléphone</t>
         </is>
       </c>
-      <c r="B71" s="4" t="n">
+      <c r="B84" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>